<commit_message>
Att Todos os resultados
</commit_message>
<xml_diff>
--- a/VNL Feminina 2025.xlsx
+++ b/VNL Feminina 2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mjunior\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{193B2670-6E0D-4629-8A7F-D6F0F42BF775}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4288B275-99FF-4688-BC8C-6E7ACB57CB84}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookPassword="CC01" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" firstSheet="1" activeTab="2" xr2:uid="{701403F6-3112-456D-B33A-FC5595D41656}"/>
@@ -857,6 +857,59 @@
     <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="18" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="12" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -927,76 +980,12 @@
     <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="17" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="12" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="103">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="2"/>
-      </font>
-    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1024,6 +1013,11 @@
           <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="2"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -1087,6 +1081,12 @@
           <bgColor rgb="FFFF9B9B"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -2217,36 +2217,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="D1" s="58" t="s">
+      <c r="D1" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="58"/>
-      <c r="F1" s="58"/>
-      <c r="G1" s="58" t="s">
+      <c r="E1" s="75"/>
+      <c r="F1" s="75"/>
+      <c r="G1" s="75" t="s">
         <v>59</v>
       </c>
-      <c r="H1" s="58"/>
-      <c r="I1" s="58"/>
-      <c r="J1" s="58"/>
-      <c r="K1" s="58"/>
-      <c r="L1" s="58"/>
-      <c r="M1" s="58" t="s">
+      <c r="H1" s="75"/>
+      <c r="I1" s="75"/>
+      <c r="J1" s="75"/>
+      <c r="K1" s="75"/>
+      <c r="L1" s="75"/>
+      <c r="M1" s="75" t="s">
         <v>60</v>
       </c>
-      <c r="N1" s="58"/>
-      <c r="O1" s="58"/>
-      <c r="P1" s="58" t="s">
+      <c r="N1" s="75"/>
+      <c r="O1" s="75"/>
+      <c r="P1" s="75" t="s">
         <v>61</v>
       </c>
-      <c r="Q1" s="58"/>
-      <c r="R1" s="58"/>
-      <c r="S1" s="58" t="s">
+      <c r="Q1" s="75"/>
+      <c r="R1" s="75"/>
+      <c r="S1" s="75" t="s">
         <v>62</v>
       </c>
-      <c r="T1" s="58"/>
-      <c r="U1" s="58"/>
-      <c r="V1" s="58"/>
-      <c r="W1" s="58"/>
+      <c r="T1" s="75"/>
+      <c r="U1" s="75"/>
+      <c r="V1" s="75"/>
+      <c r="W1" s="75"/>
       <c r="Y1" s="1" t="s">
         <v>83</v>
       </c>
@@ -2523,7 +2523,7 @@
         <v>2</v>
       </c>
       <c r="Z4" s="1">
-        <f t="shared" ref="Z4:Z20" si="9">IF(Y4&gt;=$A$16,Y4+$AA$3,Y4)</f>
+        <f t="shared" ref="Z4:Z19" si="9">IF(Y4&gt;=$A$16,Y4+$AA$3,Y4)</f>
         <v>2</v>
       </c>
     </row>
@@ -4113,36 +4113,36 @@
       </c>
     </row>
     <row r="25" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="D25" s="58" t="s">
+      <c r="D25" s="75" t="s">
         <v>14</v>
       </c>
-      <c r="E25" s="58"/>
-      <c r="F25" s="58"/>
-      <c r="G25" s="58" t="s">
+      <c r="E25" s="75"/>
+      <c r="F25" s="75"/>
+      <c r="G25" s="75" t="s">
         <v>59</v>
       </c>
-      <c r="H25" s="58"/>
-      <c r="I25" s="58"/>
-      <c r="J25" s="58"/>
-      <c r="K25" s="58"/>
-      <c r="L25" s="58"/>
-      <c r="M25" s="58" t="s">
+      <c r="H25" s="75"/>
+      <c r="I25" s="75"/>
+      <c r="J25" s="75"/>
+      <c r="K25" s="75"/>
+      <c r="L25" s="75"/>
+      <c r="M25" s="75" t="s">
         <v>60</v>
       </c>
-      <c r="N25" s="58"/>
-      <c r="O25" s="58"/>
-      <c r="P25" s="58" t="s">
+      <c r="N25" s="75"/>
+      <c r="O25" s="75"/>
+      <c r="P25" s="75" t="s">
         <v>61</v>
       </c>
-      <c r="Q25" s="58"/>
-      <c r="R25" s="58"/>
-      <c r="S25" s="58" t="s">
+      <c r="Q25" s="75"/>
+      <c r="R25" s="75"/>
+      <c r="S25" s="75" t="s">
         <v>62</v>
       </c>
-      <c r="T25" s="58"/>
-      <c r="U25" s="58"/>
-      <c r="V25" s="58"/>
-      <c r="W25" s="58"/>
+      <c r="T25" s="75"/>
+      <c r="U25" s="75"/>
+      <c r="V25" s="75"/>
+      <c r="W25" s="75"/>
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
@@ -5138,88 +5138,88 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:64" ht="15" x14ac:dyDescent="0.25">
-      <c r="B2" s="61" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
-      <c r="G2" s="61"/>
-      <c r="H2" s="61"/>
-      <c r="I2" s="61"/>
-      <c r="J2" s="61"/>
-      <c r="K2" s="61"/>
-      <c r="L2" s="61"/>
-      <c r="M2" s="61"/>
-      <c r="N2" s="61"/>
-      <c r="O2" s="61"/>
-      <c r="P2" s="61"/>
-      <c r="Q2" s="61"/>
-      <c r="R2" s="61"/>
-      <c r="S2" s="61"/>
-      <c r="T2" s="61"/>
-      <c r="U2" s="61"/>
-      <c r="V2" s="61"/>
-      <c r="W2" s="61"/>
-      <c r="X2" s="61"/>
-      <c r="Y2" s="61"/>
-      <c r="AU2" s="74" t="s">
+      <c r="B2" s="78" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="78"/>
+      <c r="N2" s="78"/>
+      <c r="O2" s="78"/>
+      <c r="P2" s="78"/>
+      <c r="Q2" s="78"/>
+      <c r="R2" s="78"/>
+      <c r="S2" s="78"/>
+      <c r="T2" s="78"/>
+      <c r="U2" s="78"/>
+      <c r="V2" s="78"/>
+      <c r="W2" s="78"/>
+      <c r="X2" s="78"/>
+      <c r="Y2" s="78"/>
+      <c r="AU2" s="91" t="s">
         <v>77</v>
       </c>
-      <c r="AV2" s="75"/>
-      <c r="AW2" s="76"/>
-      <c r="AX2" s="74" t="s">
+      <c r="AV2" s="92"/>
+      <c r="AW2" s="93"/>
+      <c r="AX2" s="91" t="s">
         <v>14</v>
       </c>
-      <c r="AY2" s="75"/>
-      <c r="AZ2" s="76"/>
-      <c r="BA2" s="74" t="s">
+      <c r="AY2" s="92"/>
+      <c r="AZ2" s="93"/>
+      <c r="BA2" s="91" t="s">
         <v>59</v>
       </c>
-      <c r="BB2" s="75"/>
-      <c r="BC2" s="75"/>
-      <c r="BD2" s="75"/>
-      <c r="BE2" s="75"/>
-      <c r="BF2" s="76"/>
-      <c r="BG2" s="74" t="s">
+      <c r="BB2" s="92"/>
+      <c r="BC2" s="92"/>
+      <c r="BD2" s="92"/>
+      <c r="BE2" s="92"/>
+      <c r="BF2" s="93"/>
+      <c r="BG2" s="91" t="s">
         <v>60</v>
       </c>
-      <c r="BH2" s="75"/>
-      <c r="BI2" s="76"/>
-      <c r="BJ2" s="74" t="s">
+      <c r="BH2" s="92"/>
+      <c r="BI2" s="93"/>
+      <c r="BJ2" s="91" t="s">
         <v>61</v>
       </c>
-      <c r="BK2" s="75"/>
-      <c r="BL2" s="76"/>
+      <c r="BK2" s="92"/>
+      <c r="BL2" s="93"/>
     </row>
     <row r="3" spans="2:64" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="B3" s="60" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60"/>
-      <c r="J3" s="60"/>
-      <c r="K3" s="60"/>
-      <c r="L3" s="60"/>
-      <c r="M3" s="60"/>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="60"/>
-      <c r="R3" s="60"/>
-      <c r="S3" s="60"/>
-      <c r="T3" s="60"/>
-      <c r="U3" s="60"/>
-      <c r="V3" s="60"/>
-      <c r="W3" s="60"/>
-      <c r="X3" s="60"/>
-      <c r="Y3" s="60"/>
+      <c r="B3" s="77" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+      <c r="I3" s="77"/>
+      <c r="J3" s="77"/>
+      <c r="K3" s="77"/>
+      <c r="L3" s="77"/>
+      <c r="M3" s="77"/>
+      <c r="N3" s="77"/>
+      <c r="O3" s="77"/>
+      <c r="P3" s="77"/>
+      <c r="Q3" s="77"/>
+      <c r="R3" s="77"/>
+      <c r="S3" s="77"/>
+      <c r="T3" s="77"/>
+      <c r="U3" s="77"/>
+      <c r="V3" s="77"/>
+      <c r="W3" s="77"/>
+      <c r="X3" s="77"/>
+      <c r="Y3" s="77"/>
       <c r="AU3" s="32" t="s">
         <v>43</v>
       </c>
@@ -5280,42 +5280,42 @@
         <v>2</v>
       </c>
       <c r="C4" s="24"/>
-      <c r="D4" s="63" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" s="63"/>
-      <c r="F4" s="63"/>
+      <c r="D4" s="80" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="80"/>
+      <c r="F4" s="80"/>
       <c r="G4" s="20"/>
-      <c r="H4" s="59" t="s">
+      <c r="H4" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="59"/>
-      <c r="J4" s="59"/>
-      <c r="K4" s="59" t="s">
+      <c r="I4" s="76"/>
+      <c r="J4" s="76"/>
+      <c r="K4" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="L4" s="59"/>
-      <c r="M4" s="59"/>
-      <c r="N4" s="59" t="s">
+      <c r="L4" s="76"/>
+      <c r="M4" s="76"/>
+      <c r="N4" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="O4" s="59"/>
-      <c r="P4" s="59"/>
-      <c r="Q4" s="59" t="s">
+      <c r="O4" s="76"/>
+      <c r="P4" s="76"/>
+      <c r="Q4" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="R4" s="59"/>
-      <c r="S4" s="59"/>
-      <c r="T4" s="59" t="s">
+      <c r="R4" s="76"/>
+      <c r="S4" s="76"/>
+      <c r="T4" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="U4" s="59"/>
-      <c r="V4" s="59"/>
-      <c r="W4" s="59" t="s">
+      <c r="U4" s="76"/>
+      <c r="V4" s="76"/>
+      <c r="W4" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="X4" s="59"/>
-      <c r="Y4" s="59"/>
+      <c r="X4" s="76"/>
+      <c r="Y4" s="76"/>
       <c r="AA4" s="4" t="s">
         <v>38</v>
       </c>
@@ -8078,32 +8078,32 @@
       </c>
     </row>
     <row r="17" spans="2:64" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="B17" s="60" t="s">
+      <c r="B17" s="77" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="60"/>
-      <c r="D17" s="60"/>
-      <c r="E17" s="62"/>
-      <c r="F17" s="60"/>
-      <c r="G17" s="60"/>
-      <c r="H17" s="60"/>
-      <c r="I17" s="60"/>
-      <c r="J17" s="60"/>
-      <c r="K17" s="60"/>
-      <c r="L17" s="60"/>
-      <c r="M17" s="60"/>
-      <c r="N17" s="60"/>
-      <c r="O17" s="60"/>
-      <c r="P17" s="60"/>
-      <c r="Q17" s="60"/>
-      <c r="R17" s="60"/>
-      <c r="S17" s="60"/>
-      <c r="T17" s="60"/>
-      <c r="U17" s="60"/>
-      <c r="V17" s="60"/>
-      <c r="W17" s="60"/>
-      <c r="X17" s="60"/>
-      <c r="Y17" s="60"/>
+      <c r="C17" s="77"/>
+      <c r="D17" s="77"/>
+      <c r="E17" s="79"/>
+      <c r="F17" s="77"/>
+      <c r="G17" s="77"/>
+      <c r="H17" s="77"/>
+      <c r="I17" s="77"/>
+      <c r="J17" s="77"/>
+      <c r="K17" s="77"/>
+      <c r="L17" s="77"/>
+      <c r="M17" s="77"/>
+      <c r="N17" s="77"/>
+      <c r="O17" s="77"/>
+      <c r="P17" s="77"/>
+      <c r="Q17" s="77"/>
+      <c r="R17" s="77"/>
+      <c r="S17" s="77"/>
+      <c r="T17" s="77"/>
+      <c r="U17" s="77"/>
+      <c r="V17" s="77"/>
+      <c r="W17" s="77"/>
+      <c r="X17" s="77"/>
+      <c r="Y17" s="77"/>
       <c r="AU17" s="31">
         <v>14</v>
       </c>
@@ -8181,42 +8181,42 @@
         <v>2</v>
       </c>
       <c r="C18" s="24"/>
-      <c r="D18" s="59" t="s">
-        <v>3</v>
-      </c>
-      <c r="E18" s="59"/>
-      <c r="F18" s="59"/>
+      <c r="D18" s="76" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" s="76"/>
+      <c r="F18" s="76"/>
       <c r="G18" s="20"/>
-      <c r="H18" s="59" t="s">
+      <c r="H18" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="I18" s="59"/>
-      <c r="J18" s="59"/>
-      <c r="K18" s="59" t="s">
+      <c r="I18" s="76"/>
+      <c r="J18" s="76"/>
+      <c r="K18" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="L18" s="59"/>
-      <c r="M18" s="59"/>
-      <c r="N18" s="59" t="s">
+      <c r="L18" s="76"/>
+      <c r="M18" s="76"/>
+      <c r="N18" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="O18" s="59"/>
-      <c r="P18" s="59"/>
-      <c r="Q18" s="59" t="s">
+      <c r="O18" s="76"/>
+      <c r="P18" s="76"/>
+      <c r="Q18" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="R18" s="59"/>
-      <c r="S18" s="59"/>
-      <c r="T18" s="59" t="s">
+      <c r="R18" s="76"/>
+      <c r="S18" s="76"/>
+      <c r="T18" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="U18" s="59"/>
-      <c r="V18" s="59"/>
-      <c r="W18" s="59" t="s">
+      <c r="U18" s="76"/>
+      <c r="V18" s="76"/>
+      <c r="W18" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="X18" s="59"/>
-      <c r="Y18" s="59"/>
+      <c r="X18" s="76"/>
+      <c r="Y18" s="76"/>
       <c r="AA18" s="4" t="s">
         <v>38</v>
       </c>
@@ -9290,10 +9290,10 @@
         <f t="shared" si="39"/>
         <v>75</v>
       </c>
-      <c r="AU23" s="73" t="s">
+      <c r="AU23" s="90" t="s">
         <v>87</v>
       </c>
-      <c r="AV23" s="73"/>
+      <c r="AV23" s="90"/>
     </row>
     <row r="24" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B24" s="18">
@@ -10344,78 +10344,78 @@
       </c>
     </row>
     <row r="31" spans="2:64" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="B31" s="60" t="s">
+      <c r="B31" s="77" t="s">
         <v>12</v>
       </c>
-      <c r="C31" s="60"/>
-      <c r="D31" s="60"/>
-      <c r="E31" s="60"/>
-      <c r="F31" s="60"/>
-      <c r="G31" s="60"/>
-      <c r="H31" s="60"/>
-      <c r="I31" s="60"/>
-      <c r="J31" s="60"/>
-      <c r="K31" s="60"/>
-      <c r="L31" s="60"/>
-      <c r="M31" s="60"/>
-      <c r="N31" s="60"/>
-      <c r="O31" s="60"/>
-      <c r="P31" s="60"/>
-      <c r="Q31" s="60"/>
-      <c r="R31" s="60"/>
-      <c r="S31" s="60"/>
-      <c r="T31" s="60"/>
-      <c r="U31" s="60"/>
-      <c r="V31" s="60"/>
-      <c r="W31" s="60"/>
-      <c r="X31" s="60"/>
-      <c r="Y31" s="60"/>
-      <c r="AU31" s="77" t="s">
+      <c r="C31" s="77"/>
+      <c r="D31" s="77"/>
+      <c r="E31" s="77"/>
+      <c r="F31" s="77"/>
+      <c r="G31" s="77"/>
+      <c r="H31" s="77"/>
+      <c r="I31" s="77"/>
+      <c r="J31" s="77"/>
+      <c r="K31" s="77"/>
+      <c r="L31" s="77"/>
+      <c r="M31" s="77"/>
+      <c r="N31" s="77"/>
+      <c r="O31" s="77"/>
+      <c r="P31" s="77"/>
+      <c r="Q31" s="77"/>
+      <c r="R31" s="77"/>
+      <c r="S31" s="77"/>
+      <c r="T31" s="77"/>
+      <c r="U31" s="77"/>
+      <c r="V31" s="77"/>
+      <c r="W31" s="77"/>
+      <c r="X31" s="77"/>
+      <c r="Y31" s="77"/>
+      <c r="AU31" s="94" t="s">
         <v>91</v>
       </c>
-      <c r="AV31" s="78"/>
+      <c r="AV31" s="95"/>
     </row>
     <row r="32" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B32" s="16" t="s">
         <v>2</v>
       </c>
       <c r="C32" s="24"/>
-      <c r="D32" s="63" t="s">
-        <v>3</v>
-      </c>
-      <c r="E32" s="63"/>
-      <c r="F32" s="63"/>
+      <c r="D32" s="80" t="s">
+        <v>3</v>
+      </c>
+      <c r="E32" s="80"/>
+      <c r="F32" s="80"/>
       <c r="G32" s="20"/>
-      <c r="H32" s="59" t="s">
+      <c r="H32" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="I32" s="59"/>
-      <c r="J32" s="59"/>
-      <c r="K32" s="59" t="s">
+      <c r="I32" s="76"/>
+      <c r="J32" s="76"/>
+      <c r="K32" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="L32" s="59"/>
-      <c r="M32" s="59"/>
-      <c r="N32" s="59" t="s">
+      <c r="L32" s="76"/>
+      <c r="M32" s="76"/>
+      <c r="N32" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="O32" s="59"/>
-      <c r="P32" s="59"/>
-      <c r="Q32" s="59" t="s">
+      <c r="O32" s="76"/>
+      <c r="P32" s="76"/>
+      <c r="Q32" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="R32" s="59"/>
-      <c r="S32" s="59"/>
-      <c r="T32" s="59" t="s">
+      <c r="R32" s="76"/>
+      <c r="S32" s="76"/>
+      <c r="T32" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="U32" s="59"/>
-      <c r="V32" s="59"/>
-      <c r="W32" s="59" t="s">
+      <c r="U32" s="76"/>
+      <c r="V32" s="76"/>
+      <c r="W32" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="X32" s="59"/>
-      <c r="Y32" s="59"/>
+      <c r="X32" s="76"/>
+      <c r="Y32" s="76"/>
       <c r="AA32" s="4" t="s">
         <v>38</v>
       </c>
@@ -10473,10 +10473,10 @@
       <c r="AT32" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="AU32" s="64" t="s">
+      <c r="AU32" s="81" t="s">
         <v>92</v>
       </c>
-      <c r="AV32" s="65"/>
+      <c r="AV32" s="82"/>
     </row>
     <row r="33" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B33" s="17">
@@ -10625,10 +10625,10 @@
         <f t="shared" ref="AT33:AT44" si="60">IF(D33&lt;F33,SUM(J33,M33,P33,S33,V33),SUM(H33,K33,N33,Q33,T33))</f>
         <v>98</v>
       </c>
-      <c r="AU33" s="66" t="s">
+      <c r="AU33" s="83" t="s">
         <v>93</v>
       </c>
-      <c r="AV33" s="67"/>
+      <c r="AV33" s="84"/>
     </row>
     <row r="34" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B34" s="17">
@@ -10773,10 +10773,10 @@
         <f t="shared" si="60"/>
         <v>76</v>
       </c>
-      <c r="AU34" s="66" t="s">
+      <c r="AU34" s="83" t="s">
         <v>94</v>
       </c>
-      <c r="AV34" s="67"/>
+      <c r="AV34" s="84"/>
     </row>
     <row r="35" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B35" s="17">
@@ -10921,10 +10921,10 @@
         <f t="shared" si="60"/>
         <v>77</v>
       </c>
-      <c r="AU35" s="66" t="s">
+      <c r="AU35" s="83" t="s">
         <v>95</v>
       </c>
-      <c r="AV35" s="67"/>
+      <c r="AV35" s="84"/>
     </row>
     <row r="36" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B36" s="17">
@@ -11073,10 +11073,10 @@
         <f t="shared" si="60"/>
         <v>99</v>
       </c>
-      <c r="AU36" s="68" t="s">
+      <c r="AU36" s="85" t="s">
         <v>96</v>
       </c>
-      <c r="AV36" s="69"/>
+      <c r="AV36" s="86"/>
     </row>
     <row r="37" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B37" s="17">
@@ -12259,88 +12259,88 @@
       </c>
     </row>
     <row r="46" spans="2:64" ht="15" x14ac:dyDescent="0.25">
-      <c r="B46" s="61" t="s">
+      <c r="B46" s="78" t="s">
         <v>67</v>
       </c>
-      <c r="C46" s="61"/>
-      <c r="D46" s="61"/>
-      <c r="E46" s="61"/>
-      <c r="F46" s="61"/>
-      <c r="G46" s="61"/>
-      <c r="H46" s="61"/>
-      <c r="I46" s="61"/>
-      <c r="J46" s="61"/>
-      <c r="K46" s="61"/>
-      <c r="L46" s="61"/>
-      <c r="M46" s="61"/>
-      <c r="N46" s="61"/>
-      <c r="O46" s="61"/>
-      <c r="P46" s="61"/>
-      <c r="Q46" s="61"/>
-      <c r="R46" s="61"/>
-      <c r="S46" s="61"/>
-      <c r="T46" s="61"/>
-      <c r="U46" s="61"/>
-      <c r="V46" s="61"/>
-      <c r="W46" s="61"/>
-      <c r="X46" s="61"/>
-      <c r="Y46" s="61"/>
-      <c r="AU46" s="70" t="s">
+      <c r="C46" s="78"/>
+      <c r="D46" s="78"/>
+      <c r="E46" s="78"/>
+      <c r="F46" s="78"/>
+      <c r="G46" s="78"/>
+      <c r="H46" s="78"/>
+      <c r="I46" s="78"/>
+      <c r="J46" s="78"/>
+      <c r="K46" s="78"/>
+      <c r="L46" s="78"/>
+      <c r="M46" s="78"/>
+      <c r="N46" s="78"/>
+      <c r="O46" s="78"/>
+      <c r="P46" s="78"/>
+      <c r="Q46" s="78"/>
+      <c r="R46" s="78"/>
+      <c r="S46" s="78"/>
+      <c r="T46" s="78"/>
+      <c r="U46" s="78"/>
+      <c r="V46" s="78"/>
+      <c r="W46" s="78"/>
+      <c r="X46" s="78"/>
+      <c r="Y46" s="78"/>
+      <c r="AU46" s="87" t="s">
         <v>77</v>
       </c>
-      <c r="AV46" s="71"/>
-      <c r="AW46" s="72"/>
-      <c r="AX46" s="70" t="s">
+      <c r="AV46" s="88"/>
+      <c r="AW46" s="89"/>
+      <c r="AX46" s="87" t="s">
         <v>14</v>
       </c>
-      <c r="AY46" s="71"/>
-      <c r="AZ46" s="72"/>
-      <c r="BA46" s="70" t="s">
+      <c r="AY46" s="88"/>
+      <c r="AZ46" s="89"/>
+      <c r="BA46" s="87" t="s">
         <v>59</v>
       </c>
-      <c r="BB46" s="71"/>
-      <c r="BC46" s="71"/>
-      <c r="BD46" s="71"/>
-      <c r="BE46" s="71"/>
-      <c r="BF46" s="72"/>
-      <c r="BG46" s="70" t="s">
+      <c r="BB46" s="88"/>
+      <c r="BC46" s="88"/>
+      <c r="BD46" s="88"/>
+      <c r="BE46" s="88"/>
+      <c r="BF46" s="89"/>
+      <c r="BG46" s="87" t="s">
         <v>60</v>
       </c>
-      <c r="BH46" s="71"/>
-      <c r="BI46" s="72"/>
-      <c r="BJ46" s="70" t="s">
+      <c r="BH46" s="88"/>
+      <c r="BI46" s="89"/>
+      <c r="BJ46" s="87" t="s">
         <v>61</v>
       </c>
-      <c r="BK46" s="71"/>
-      <c r="BL46" s="72"/>
+      <c r="BK46" s="88"/>
+      <c r="BL46" s="89"/>
     </row>
     <row r="47" spans="2:64" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="B47" s="60" t="s">
+      <c r="B47" s="77" t="s">
         <v>13</v>
       </c>
-      <c r="C47" s="60"/>
-      <c r="D47" s="60"/>
-      <c r="E47" s="60"/>
-      <c r="F47" s="60"/>
-      <c r="G47" s="60"/>
-      <c r="H47" s="60"/>
-      <c r="I47" s="60"/>
-      <c r="J47" s="60"/>
-      <c r="K47" s="60"/>
-      <c r="L47" s="60"/>
-      <c r="M47" s="60"/>
-      <c r="N47" s="60"/>
-      <c r="O47" s="60"/>
-      <c r="P47" s="60"/>
-      <c r="Q47" s="60"/>
-      <c r="R47" s="60"/>
-      <c r="S47" s="60"/>
-      <c r="T47" s="60"/>
-      <c r="U47" s="60"/>
-      <c r="V47" s="60"/>
-      <c r="W47" s="60"/>
-      <c r="X47" s="60"/>
-      <c r="Y47" s="60"/>
+      <c r="C47" s="77"/>
+      <c r="D47" s="77"/>
+      <c r="E47" s="77"/>
+      <c r="F47" s="77"/>
+      <c r="G47" s="77"/>
+      <c r="H47" s="77"/>
+      <c r="I47" s="77"/>
+      <c r="J47" s="77"/>
+      <c r="K47" s="77"/>
+      <c r="L47" s="77"/>
+      <c r="M47" s="77"/>
+      <c r="N47" s="77"/>
+      <c r="O47" s="77"/>
+      <c r="P47" s="77"/>
+      <c r="Q47" s="77"/>
+      <c r="R47" s="77"/>
+      <c r="S47" s="77"/>
+      <c r="T47" s="77"/>
+      <c r="U47" s="77"/>
+      <c r="V47" s="77"/>
+      <c r="W47" s="77"/>
+      <c r="X47" s="77"/>
+      <c r="Y47" s="77"/>
       <c r="AU47" s="32" t="s">
         <v>43</v>
       </c>
@@ -12401,42 +12401,42 @@
         <v>2</v>
       </c>
       <c r="C48" s="24"/>
-      <c r="D48" s="63" t="s">
-        <v>3</v>
-      </c>
-      <c r="E48" s="63"/>
-      <c r="F48" s="63"/>
+      <c r="D48" s="80" t="s">
+        <v>3</v>
+      </c>
+      <c r="E48" s="80"/>
+      <c r="F48" s="80"/>
       <c r="G48" s="20"/>
-      <c r="H48" s="59" t="s">
+      <c r="H48" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="I48" s="59"/>
-      <c r="J48" s="59"/>
-      <c r="K48" s="59" t="s">
+      <c r="I48" s="76"/>
+      <c r="J48" s="76"/>
+      <c r="K48" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="L48" s="59"/>
-      <c r="M48" s="59"/>
-      <c r="N48" s="59" t="s">
+      <c r="L48" s="76"/>
+      <c r="M48" s="76"/>
+      <c r="N48" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="O48" s="59"/>
-      <c r="P48" s="59"/>
-      <c r="Q48" s="59" t="s">
+      <c r="O48" s="76"/>
+      <c r="P48" s="76"/>
+      <c r="Q48" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="R48" s="59"/>
-      <c r="S48" s="59"/>
-      <c r="T48" s="59" t="s">
+      <c r="R48" s="76"/>
+      <c r="S48" s="76"/>
+      <c r="T48" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="U48" s="59"/>
-      <c r="V48" s="59"/>
-      <c r="W48" s="59" t="s">
+      <c r="U48" s="76"/>
+      <c r="V48" s="76"/>
+      <c r="W48" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="X48" s="59"/>
-      <c r="Y48" s="59"/>
+      <c r="X48" s="76"/>
+      <c r="Y48" s="76"/>
       <c r="AA48" s="4" t="s">
         <v>38</v>
       </c>
@@ -15183,32 +15183,32 @@
       </c>
     </row>
     <row r="61" spans="2:64" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="B61" s="60" t="s">
+      <c r="B61" s="77" t="s">
         <v>68</v>
       </c>
-      <c r="C61" s="60"/>
-      <c r="D61" s="60"/>
-      <c r="E61" s="62"/>
-      <c r="F61" s="60"/>
-      <c r="G61" s="60"/>
-      <c r="H61" s="60"/>
-      <c r="I61" s="60"/>
-      <c r="J61" s="60"/>
-      <c r="K61" s="60"/>
-      <c r="L61" s="60"/>
-      <c r="M61" s="60"/>
-      <c r="N61" s="60"/>
-      <c r="O61" s="60"/>
-      <c r="P61" s="60"/>
-      <c r="Q61" s="60"/>
-      <c r="R61" s="60"/>
-      <c r="S61" s="60"/>
-      <c r="T61" s="60"/>
-      <c r="U61" s="60"/>
-      <c r="V61" s="60"/>
-      <c r="W61" s="60"/>
-      <c r="X61" s="60"/>
-      <c r="Y61" s="60"/>
+      <c r="C61" s="77"/>
+      <c r="D61" s="77"/>
+      <c r="E61" s="79"/>
+      <c r="F61" s="77"/>
+      <c r="G61" s="77"/>
+      <c r="H61" s="77"/>
+      <c r="I61" s="77"/>
+      <c r="J61" s="77"/>
+      <c r="K61" s="77"/>
+      <c r="L61" s="77"/>
+      <c r="M61" s="77"/>
+      <c r="N61" s="77"/>
+      <c r="O61" s="77"/>
+      <c r="P61" s="77"/>
+      <c r="Q61" s="77"/>
+      <c r="R61" s="77"/>
+      <c r="S61" s="77"/>
+      <c r="T61" s="77"/>
+      <c r="U61" s="77"/>
+      <c r="V61" s="77"/>
+      <c r="W61" s="77"/>
+      <c r="X61" s="77"/>
+      <c r="Y61" s="77"/>
       <c r="AU61" s="31">
         <v>14</v>
       </c>
@@ -15286,42 +15286,42 @@
         <v>2</v>
       </c>
       <c r="C62" s="24"/>
-      <c r="D62" s="59" t="s">
-        <v>3</v>
-      </c>
-      <c r="E62" s="59"/>
-      <c r="F62" s="59"/>
+      <c r="D62" s="76" t="s">
+        <v>3</v>
+      </c>
+      <c r="E62" s="76"/>
+      <c r="F62" s="76"/>
       <c r="G62" s="20"/>
-      <c r="H62" s="59" t="s">
+      <c r="H62" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="I62" s="59"/>
-      <c r="J62" s="59"/>
-      <c r="K62" s="59" t="s">
+      <c r="I62" s="76"/>
+      <c r="J62" s="76"/>
+      <c r="K62" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="L62" s="59"/>
-      <c r="M62" s="59"/>
-      <c r="N62" s="59" t="s">
+      <c r="L62" s="76"/>
+      <c r="M62" s="76"/>
+      <c r="N62" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="O62" s="59"/>
-      <c r="P62" s="59"/>
-      <c r="Q62" s="59" t="s">
+      <c r="O62" s="76"/>
+      <c r="P62" s="76"/>
+      <c r="Q62" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="R62" s="59"/>
-      <c r="S62" s="59"/>
-      <c r="T62" s="59" t="s">
+      <c r="R62" s="76"/>
+      <c r="S62" s="76"/>
+      <c r="T62" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="U62" s="59"/>
-      <c r="V62" s="59"/>
-      <c r="W62" s="59" t="s">
+      <c r="U62" s="76"/>
+      <c r="V62" s="76"/>
+      <c r="W62" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="X62" s="59"/>
-      <c r="Y62" s="59"/>
+      <c r="X62" s="76"/>
+      <c r="Y62" s="76"/>
       <c r="AA62" s="4" t="s">
         <v>38</v>
       </c>
@@ -16411,10 +16411,10 @@
         <f t="shared" si="102"/>
         <v>112</v>
       </c>
-      <c r="AU67" s="73" t="s">
+      <c r="AU67" s="90" t="s">
         <v>87</v>
       </c>
-      <c r="AV67" s="73"/>
+      <c r="AV67" s="90"/>
     </row>
     <row r="68" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B68" s="18">
@@ -17457,78 +17457,78 @@
       </c>
     </row>
     <row r="75" spans="2:64" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="B75" s="60" t="s">
+      <c r="B75" s="77" t="s">
         <v>69</v>
       </c>
-      <c r="C75" s="60"/>
-      <c r="D75" s="60"/>
-      <c r="E75" s="60"/>
-      <c r="F75" s="60"/>
-      <c r="G75" s="60"/>
-      <c r="H75" s="60"/>
-      <c r="I75" s="60"/>
-      <c r="J75" s="60"/>
-      <c r="K75" s="60"/>
-      <c r="L75" s="60"/>
-      <c r="M75" s="60"/>
-      <c r="N75" s="60"/>
-      <c r="O75" s="60"/>
-      <c r="P75" s="60"/>
-      <c r="Q75" s="60"/>
-      <c r="R75" s="60"/>
-      <c r="S75" s="60"/>
-      <c r="T75" s="60"/>
-      <c r="U75" s="60"/>
-      <c r="V75" s="60"/>
-      <c r="W75" s="60"/>
-      <c r="X75" s="60"/>
-      <c r="Y75" s="60"/>
-      <c r="AU75" s="77" t="s">
+      <c r="C75" s="77"/>
+      <c r="D75" s="77"/>
+      <c r="E75" s="77"/>
+      <c r="F75" s="77"/>
+      <c r="G75" s="77"/>
+      <c r="H75" s="77"/>
+      <c r="I75" s="77"/>
+      <c r="J75" s="77"/>
+      <c r="K75" s="77"/>
+      <c r="L75" s="77"/>
+      <c r="M75" s="77"/>
+      <c r="N75" s="77"/>
+      <c r="O75" s="77"/>
+      <c r="P75" s="77"/>
+      <c r="Q75" s="77"/>
+      <c r="R75" s="77"/>
+      <c r="S75" s="77"/>
+      <c r="T75" s="77"/>
+      <c r="U75" s="77"/>
+      <c r="V75" s="77"/>
+      <c r="W75" s="77"/>
+      <c r="X75" s="77"/>
+      <c r="Y75" s="77"/>
+      <c r="AU75" s="94" t="s">
         <v>91</v>
       </c>
-      <c r="AV75" s="78"/>
+      <c r="AV75" s="95"/>
     </row>
     <row r="76" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B76" s="16" t="s">
         <v>2</v>
       </c>
       <c r="C76" s="24"/>
-      <c r="D76" s="63" t="s">
-        <v>3</v>
-      </c>
-      <c r="E76" s="63"/>
-      <c r="F76" s="63"/>
+      <c r="D76" s="80" t="s">
+        <v>3</v>
+      </c>
+      <c r="E76" s="80"/>
+      <c r="F76" s="80"/>
       <c r="G76" s="20"/>
-      <c r="H76" s="59" t="s">
+      <c r="H76" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="I76" s="59"/>
-      <c r="J76" s="59"/>
-      <c r="K76" s="59" t="s">
+      <c r="I76" s="76"/>
+      <c r="J76" s="76"/>
+      <c r="K76" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="L76" s="59"/>
-      <c r="M76" s="59"/>
-      <c r="N76" s="59" t="s">
+      <c r="L76" s="76"/>
+      <c r="M76" s="76"/>
+      <c r="N76" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="O76" s="59"/>
-      <c r="P76" s="59"/>
-      <c r="Q76" s="59" t="s">
+      <c r="O76" s="76"/>
+      <c r="P76" s="76"/>
+      <c r="Q76" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="R76" s="59"/>
-      <c r="S76" s="59"/>
-      <c r="T76" s="59" t="s">
+      <c r="R76" s="76"/>
+      <c r="S76" s="76"/>
+      <c r="T76" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="U76" s="59"/>
-      <c r="V76" s="59"/>
-      <c r="W76" s="59" t="s">
+      <c r="U76" s="76"/>
+      <c r="V76" s="76"/>
+      <c r="W76" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="X76" s="59"/>
-      <c r="Y76" s="59"/>
+      <c r="X76" s="76"/>
+      <c r="Y76" s="76"/>
       <c r="AA76" s="4" t="s">
         <v>38</v>
       </c>
@@ -17586,10 +17586,10 @@
       <c r="AT76" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="AU76" s="64" t="s">
+      <c r="AU76" s="81" t="s">
         <v>92</v>
       </c>
-      <c r="AV76" s="65"/>
+      <c r="AV76" s="82"/>
     </row>
     <row r="77" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B77" s="17">
@@ -17742,10 +17742,10 @@
         <f t="shared" ref="AT77:AT88" si="123">IF(D77&lt;F77,SUM(J77,M77,P77,S77,V77),SUM(H77,K77,N77,Q77,T77))</f>
         <v>112</v>
       </c>
-      <c r="AU77" s="66" t="s">
+      <c r="AU77" s="83" t="s">
         <v>93</v>
       </c>
-      <c r="AV77" s="67"/>
+      <c r="AV77" s="84"/>
     </row>
     <row r="78" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B78" s="17">
@@ -17898,10 +17898,10 @@
         <f t="shared" si="123"/>
         <v>99</v>
       </c>
-      <c r="AU78" s="66" t="s">
+      <c r="AU78" s="83" t="s">
         <v>94</v>
       </c>
-      <c r="AV78" s="67"/>
+      <c r="AV78" s="84"/>
     </row>
     <row r="79" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B79" s="17">
@@ -18054,10 +18054,10 @@
         <f t="shared" si="123"/>
         <v>109</v>
       </c>
-      <c r="AU79" s="66" t="s">
+      <c r="AU79" s="83" t="s">
         <v>95</v>
       </c>
-      <c r="AV79" s="67"/>
+      <c r="AV79" s="84"/>
     </row>
     <row r="80" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B80" s="17">
@@ -18206,10 +18206,10 @@
         <f t="shared" si="123"/>
         <v>95</v>
       </c>
-      <c r="AU80" s="68" t="s">
+      <c r="AU80" s="85" t="s">
         <v>96</v>
       </c>
-      <c r="AV80" s="69"/>
+      <c r="AV80" s="86"/>
     </row>
     <row r="81" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B81" s="17">
@@ -19396,88 +19396,88 @@
       </c>
     </row>
     <row r="90" spans="2:64" ht="15" x14ac:dyDescent="0.25">
-      <c r="B90" s="61" t="s">
+      <c r="B90" s="78" t="s">
         <v>70</v>
       </c>
-      <c r="C90" s="61"/>
-      <c r="D90" s="61"/>
-      <c r="E90" s="61"/>
-      <c r="F90" s="61"/>
-      <c r="G90" s="61"/>
-      <c r="H90" s="61"/>
-      <c r="I90" s="61"/>
-      <c r="J90" s="61"/>
-      <c r="K90" s="61"/>
-      <c r="L90" s="61"/>
-      <c r="M90" s="61"/>
-      <c r="N90" s="61"/>
-      <c r="O90" s="61"/>
-      <c r="P90" s="61"/>
-      <c r="Q90" s="61"/>
-      <c r="R90" s="61"/>
-      <c r="S90" s="61"/>
-      <c r="T90" s="61"/>
-      <c r="U90" s="61"/>
-      <c r="V90" s="61"/>
-      <c r="W90" s="61"/>
-      <c r="X90" s="61"/>
-      <c r="Y90" s="61"/>
-      <c r="AU90" s="70" t="s">
+      <c r="C90" s="78"/>
+      <c r="D90" s="78"/>
+      <c r="E90" s="78"/>
+      <c r="F90" s="78"/>
+      <c r="G90" s="78"/>
+      <c r="H90" s="78"/>
+      <c r="I90" s="78"/>
+      <c r="J90" s="78"/>
+      <c r="K90" s="78"/>
+      <c r="L90" s="78"/>
+      <c r="M90" s="78"/>
+      <c r="N90" s="78"/>
+      <c r="O90" s="78"/>
+      <c r="P90" s="78"/>
+      <c r="Q90" s="78"/>
+      <c r="R90" s="78"/>
+      <c r="S90" s="78"/>
+      <c r="T90" s="78"/>
+      <c r="U90" s="78"/>
+      <c r="V90" s="78"/>
+      <c r="W90" s="78"/>
+      <c r="X90" s="78"/>
+      <c r="Y90" s="78"/>
+      <c r="AU90" s="87" t="s">
         <v>77</v>
       </c>
-      <c r="AV90" s="71"/>
-      <c r="AW90" s="72"/>
-      <c r="AX90" s="70" t="s">
+      <c r="AV90" s="88"/>
+      <c r="AW90" s="89"/>
+      <c r="AX90" s="87" t="s">
         <v>14</v>
       </c>
-      <c r="AY90" s="71"/>
-      <c r="AZ90" s="72"/>
-      <c r="BA90" s="70" t="s">
+      <c r="AY90" s="88"/>
+      <c r="AZ90" s="89"/>
+      <c r="BA90" s="87" t="s">
         <v>59</v>
       </c>
-      <c r="BB90" s="71"/>
-      <c r="BC90" s="71"/>
-      <c r="BD90" s="71"/>
-      <c r="BE90" s="71"/>
-      <c r="BF90" s="72"/>
-      <c r="BG90" s="70" t="s">
+      <c r="BB90" s="88"/>
+      <c r="BC90" s="88"/>
+      <c r="BD90" s="88"/>
+      <c r="BE90" s="88"/>
+      <c r="BF90" s="89"/>
+      <c r="BG90" s="87" t="s">
         <v>60</v>
       </c>
-      <c r="BH90" s="71"/>
-      <c r="BI90" s="72"/>
-      <c r="BJ90" s="70" t="s">
+      <c r="BH90" s="88"/>
+      <c r="BI90" s="89"/>
+      <c r="BJ90" s="87" t="s">
         <v>61</v>
       </c>
-      <c r="BK90" s="71"/>
-      <c r="BL90" s="72"/>
+      <c r="BK90" s="88"/>
+      <c r="BL90" s="89"/>
     </row>
     <row r="91" spans="2:64" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="B91" s="60" t="s">
+      <c r="B91" s="77" t="s">
         <v>71</v>
       </c>
-      <c r="C91" s="60"/>
-      <c r="D91" s="60"/>
-      <c r="E91" s="60"/>
-      <c r="F91" s="60"/>
-      <c r="G91" s="60"/>
-      <c r="H91" s="60"/>
-      <c r="I91" s="60"/>
-      <c r="J91" s="60"/>
-      <c r="K91" s="60"/>
-      <c r="L91" s="60"/>
-      <c r="M91" s="60"/>
-      <c r="N91" s="60"/>
-      <c r="O91" s="60"/>
-      <c r="P91" s="60"/>
-      <c r="Q91" s="60"/>
-      <c r="R91" s="60"/>
-      <c r="S91" s="60"/>
-      <c r="T91" s="60"/>
-      <c r="U91" s="60"/>
-      <c r="V91" s="60"/>
-      <c r="W91" s="60"/>
-      <c r="X91" s="60"/>
-      <c r="Y91" s="60"/>
+      <c r="C91" s="77"/>
+      <c r="D91" s="77"/>
+      <c r="E91" s="77"/>
+      <c r="F91" s="77"/>
+      <c r="G91" s="77"/>
+      <c r="H91" s="77"/>
+      <c r="I91" s="77"/>
+      <c r="J91" s="77"/>
+      <c r="K91" s="77"/>
+      <c r="L91" s="77"/>
+      <c r="M91" s="77"/>
+      <c r="N91" s="77"/>
+      <c r="O91" s="77"/>
+      <c r="P91" s="77"/>
+      <c r="Q91" s="77"/>
+      <c r="R91" s="77"/>
+      <c r="S91" s="77"/>
+      <c r="T91" s="77"/>
+      <c r="U91" s="77"/>
+      <c r="V91" s="77"/>
+      <c r="W91" s="77"/>
+      <c r="X91" s="77"/>
+      <c r="Y91" s="77"/>
       <c r="AU91" s="32" t="s">
         <v>43</v>
       </c>
@@ -19538,42 +19538,42 @@
         <v>2</v>
       </c>
       <c r="C92" s="24"/>
-      <c r="D92" s="63" t="s">
-        <v>3</v>
-      </c>
-      <c r="E92" s="63"/>
-      <c r="F92" s="63"/>
+      <c r="D92" s="80" t="s">
+        <v>3</v>
+      </c>
+      <c r="E92" s="80"/>
+      <c r="F92" s="80"/>
       <c r="G92" s="20"/>
-      <c r="H92" s="59" t="s">
+      <c r="H92" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="I92" s="59"/>
-      <c r="J92" s="59"/>
-      <c r="K92" s="59" t="s">
+      <c r="I92" s="76"/>
+      <c r="J92" s="76"/>
+      <c r="K92" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="L92" s="59"/>
-      <c r="M92" s="59"/>
-      <c r="N92" s="59" t="s">
+      <c r="L92" s="76"/>
+      <c r="M92" s="76"/>
+      <c r="N92" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="O92" s="59"/>
-      <c r="P92" s="59"/>
-      <c r="Q92" s="59" t="s">
+      <c r="O92" s="76"/>
+      <c r="P92" s="76"/>
+      <c r="Q92" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="R92" s="59"/>
-      <c r="S92" s="59"/>
-      <c r="T92" s="59" t="s">
+      <c r="R92" s="76"/>
+      <c r="S92" s="76"/>
+      <c r="T92" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="U92" s="59"/>
-      <c r="V92" s="59"/>
-      <c r="W92" s="59" t="s">
+      <c r="U92" s="76"/>
+      <c r="V92" s="76"/>
+      <c r="W92" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="X92" s="59"/>
-      <c r="Y92" s="59"/>
+      <c r="X92" s="76"/>
+      <c r="Y92" s="76"/>
       <c r="AA92" s="4" t="s">
         <v>38</v>
       </c>
@@ -22316,32 +22316,32 @@
       </c>
     </row>
     <row r="105" spans="2:64" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="B105" s="60" t="s">
+      <c r="B105" s="77" t="s">
         <v>72</v>
       </c>
-      <c r="C105" s="60"/>
-      <c r="D105" s="60"/>
-      <c r="E105" s="62"/>
-      <c r="F105" s="60"/>
-      <c r="G105" s="60"/>
-      <c r="H105" s="60"/>
-      <c r="I105" s="60"/>
-      <c r="J105" s="60"/>
-      <c r="K105" s="60"/>
-      <c r="L105" s="60"/>
-      <c r="M105" s="60"/>
-      <c r="N105" s="60"/>
-      <c r="O105" s="60"/>
-      <c r="P105" s="60"/>
-      <c r="Q105" s="60"/>
-      <c r="R105" s="60"/>
-      <c r="S105" s="60"/>
-      <c r="T105" s="60"/>
-      <c r="U105" s="60"/>
-      <c r="V105" s="60"/>
-      <c r="W105" s="60"/>
-      <c r="X105" s="60"/>
-      <c r="Y105" s="60"/>
+      <c r="C105" s="77"/>
+      <c r="D105" s="77"/>
+      <c r="E105" s="79"/>
+      <c r="F105" s="77"/>
+      <c r="G105" s="77"/>
+      <c r="H105" s="77"/>
+      <c r="I105" s="77"/>
+      <c r="J105" s="77"/>
+      <c r="K105" s="77"/>
+      <c r="L105" s="77"/>
+      <c r="M105" s="77"/>
+      <c r="N105" s="77"/>
+      <c r="O105" s="77"/>
+      <c r="P105" s="77"/>
+      <c r="Q105" s="77"/>
+      <c r="R105" s="77"/>
+      <c r="S105" s="77"/>
+      <c r="T105" s="77"/>
+      <c r="U105" s="77"/>
+      <c r="V105" s="77"/>
+      <c r="W105" s="77"/>
+      <c r="X105" s="77"/>
+      <c r="Y105" s="77"/>
       <c r="AU105" s="31">
         <v>14</v>
       </c>
@@ -22419,42 +22419,42 @@
         <v>2</v>
       </c>
       <c r="C106" s="24"/>
-      <c r="D106" s="59" t="s">
-        <v>3</v>
-      </c>
-      <c r="E106" s="59"/>
-      <c r="F106" s="59"/>
+      <c r="D106" s="76" t="s">
+        <v>3</v>
+      </c>
+      <c r="E106" s="76"/>
+      <c r="F106" s="76"/>
       <c r="G106" s="20"/>
-      <c r="H106" s="59" t="s">
+      <c r="H106" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="I106" s="59"/>
-      <c r="J106" s="59"/>
-      <c r="K106" s="59" t="s">
+      <c r="I106" s="76"/>
+      <c r="J106" s="76"/>
+      <c r="K106" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="L106" s="59"/>
-      <c r="M106" s="59"/>
-      <c r="N106" s="59" t="s">
+      <c r="L106" s="76"/>
+      <c r="M106" s="76"/>
+      <c r="N106" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="O106" s="59"/>
-      <c r="P106" s="59"/>
-      <c r="Q106" s="59" t="s">
+      <c r="O106" s="76"/>
+      <c r="P106" s="76"/>
+      <c r="Q106" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="R106" s="59"/>
-      <c r="S106" s="59"/>
-      <c r="T106" s="59" t="s">
+      <c r="R106" s="76"/>
+      <c r="S106" s="76"/>
+      <c r="T106" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="U106" s="59"/>
-      <c r="V106" s="59"/>
-      <c r="W106" s="59" t="s">
+      <c r="U106" s="76"/>
+      <c r="V106" s="76"/>
+      <c r="W106" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="X106" s="59"/>
-      <c r="Y106" s="59"/>
+      <c r="X106" s="76"/>
+      <c r="Y106" s="76"/>
       <c r="AA106" s="4" t="s">
         <v>38</v>
       </c>
@@ -23544,10 +23544,10 @@
         <f t="shared" si="165"/>
         <v>98</v>
       </c>
-      <c r="AU111" s="73" t="s">
+      <c r="AU111" s="90" t="s">
         <v>87</v>
       </c>
-      <c r="AV111" s="73"/>
+      <c r="AV111" s="90"/>
     </row>
     <row r="112" spans="2:64" x14ac:dyDescent="0.25">
       <c r="B112" s="18">
@@ -24610,78 +24610,78 @@
       </c>
     </row>
     <row r="119" spans="2:48" ht="14.25" x14ac:dyDescent="0.25">
-      <c r="B119" s="60" t="s">
+      <c r="B119" s="77" t="s">
         <v>73</v>
       </c>
-      <c r="C119" s="60"/>
-      <c r="D119" s="60"/>
-      <c r="E119" s="60"/>
-      <c r="F119" s="60"/>
-      <c r="G119" s="60"/>
-      <c r="H119" s="60"/>
-      <c r="I119" s="60"/>
-      <c r="J119" s="60"/>
-      <c r="K119" s="60"/>
-      <c r="L119" s="60"/>
-      <c r="M119" s="60"/>
-      <c r="N119" s="60"/>
-      <c r="O119" s="60"/>
-      <c r="P119" s="60"/>
-      <c r="Q119" s="60"/>
-      <c r="R119" s="60"/>
-      <c r="S119" s="60"/>
-      <c r="T119" s="60"/>
-      <c r="U119" s="60"/>
-      <c r="V119" s="60"/>
-      <c r="W119" s="60"/>
-      <c r="X119" s="60"/>
-      <c r="Y119" s="60"/>
-      <c r="AU119" s="77" t="s">
+      <c r="C119" s="77"/>
+      <c r="D119" s="77"/>
+      <c r="E119" s="77"/>
+      <c r="F119" s="77"/>
+      <c r="G119" s="77"/>
+      <c r="H119" s="77"/>
+      <c r="I119" s="77"/>
+      <c r="J119" s="77"/>
+      <c r="K119" s="77"/>
+      <c r="L119" s="77"/>
+      <c r="M119" s="77"/>
+      <c r="N119" s="77"/>
+      <c r="O119" s="77"/>
+      <c r="P119" s="77"/>
+      <c r="Q119" s="77"/>
+      <c r="R119" s="77"/>
+      <c r="S119" s="77"/>
+      <c r="T119" s="77"/>
+      <c r="U119" s="77"/>
+      <c r="V119" s="77"/>
+      <c r="W119" s="77"/>
+      <c r="X119" s="77"/>
+      <c r="Y119" s="77"/>
+      <c r="AU119" s="94" t="s">
         <v>91</v>
       </c>
-      <c r="AV119" s="78"/>
+      <c r="AV119" s="95"/>
     </row>
     <row r="120" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B120" s="16" t="s">
         <v>2</v>
       </c>
       <c r="C120" s="24"/>
-      <c r="D120" s="63" t="s">
-        <v>3</v>
-      </c>
-      <c r="E120" s="63"/>
-      <c r="F120" s="63"/>
+      <c r="D120" s="80" t="s">
+        <v>3</v>
+      </c>
+      <c r="E120" s="80"/>
+      <c r="F120" s="80"/>
       <c r="G120" s="20"/>
-      <c r="H120" s="59" t="s">
+      <c r="H120" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="I120" s="59"/>
-      <c r="J120" s="59"/>
-      <c r="K120" s="59" t="s">
+      <c r="I120" s="76"/>
+      <c r="J120" s="76"/>
+      <c r="K120" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="L120" s="59"/>
-      <c r="M120" s="59"/>
-      <c r="N120" s="59" t="s">
+      <c r="L120" s="76"/>
+      <c r="M120" s="76"/>
+      <c r="N120" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="O120" s="59"/>
-      <c r="P120" s="59"/>
-      <c r="Q120" s="59" t="s">
+      <c r="O120" s="76"/>
+      <c r="P120" s="76"/>
+      <c r="Q120" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="R120" s="59"/>
-      <c r="S120" s="59"/>
-      <c r="T120" s="59" t="s">
+      <c r="R120" s="76"/>
+      <c r="S120" s="76"/>
+      <c r="T120" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="U120" s="59"/>
-      <c r="V120" s="59"/>
-      <c r="W120" s="59" t="s">
+      <c r="U120" s="76"/>
+      <c r="V120" s="76"/>
+      <c r="W120" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="X120" s="59"/>
-      <c r="Y120" s="59"/>
+      <c r="X120" s="76"/>
+      <c r="Y120" s="76"/>
       <c r="AA120" s="4" t="s">
         <v>38</v>
       </c>
@@ -24739,10 +24739,10 @@
       <c r="AT120" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="AU120" s="64" t="s">
+      <c r="AU120" s="81" t="s">
         <v>92</v>
       </c>
-      <c r="AV120" s="65"/>
+      <c r="AV120" s="82"/>
     </row>
     <row r="121" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B121" s="17">
@@ -24891,10 +24891,10 @@
         <f t="shared" ref="AT121:AT132" si="186">IF(D121&lt;F121,SUM(J121,M121,P121,S121,V121),SUM(H121,K121,N121,Q121,T121))</f>
         <v>102</v>
       </c>
-      <c r="AU121" s="66" t="s">
+      <c r="AU121" s="83" t="s">
         <v>93</v>
       </c>
-      <c r="AV121" s="67"/>
+      <c r="AV121" s="84"/>
     </row>
     <row r="122" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B122" s="17">
@@ -25043,10 +25043,10 @@
         <f t="shared" si="186"/>
         <v>96</v>
       </c>
-      <c r="AU122" s="66" t="s">
+      <c r="AU122" s="83" t="s">
         <v>94</v>
       </c>
-      <c r="AV122" s="67"/>
+      <c r="AV122" s="84"/>
     </row>
     <row r="123" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B123" s="17">
@@ -25191,10 +25191,10 @@
         <f t="shared" si="186"/>
         <v>75</v>
       </c>
-      <c r="AU123" s="66" t="s">
+      <c r="AU123" s="83" t="s">
         <v>95</v>
       </c>
-      <c r="AV123" s="67"/>
+      <c r="AV123" s="84"/>
     </row>
     <row r="124" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B124" s="17">
@@ -25347,10 +25347,10 @@
         <f t="shared" si="186"/>
         <v>105</v>
       </c>
-      <c r="AU124" s="68" t="s">
+      <c r="AU124" s="85" t="s">
         <v>96</v>
       </c>
-      <c r="AV124" s="69"/>
+      <c r="AV124" s="86"/>
     </row>
     <row r="125" spans="2:48" x14ac:dyDescent="0.25">
       <c r="B125" s="17">
@@ -27183,101 +27183,101 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:65" ht="15" x14ac:dyDescent="0.25">
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="78" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="61"/>
-      <c r="D2" s="61"/>
-      <c r="E2" s="61"/>
-      <c r="F2" s="61"/>
-      <c r="G2" s="61"/>
-      <c r="H2" s="61"/>
-      <c r="I2" s="61"/>
-      <c r="J2" s="61"/>
-      <c r="K2" s="61"/>
-      <c r="L2" s="61"/>
-      <c r="M2" s="61"/>
-      <c r="N2" s="61"/>
-      <c r="O2" s="61"/>
-      <c r="P2" s="61"/>
-      <c r="Q2" s="61"/>
-      <c r="R2" s="61"/>
-      <c r="S2" s="61"/>
-      <c r="T2" s="61"/>
-      <c r="U2" s="61"/>
-      <c r="V2" s="61"/>
-      <c r="W2" s="61"/>
-      <c r="X2" s="61"/>
-      <c r="Y2" s="61"/>
-      <c r="AU2" s="74" t="s">
+      <c r="C2" s="78"/>
+      <c r="D2" s="78"/>
+      <c r="E2" s="78"/>
+      <c r="F2" s="78"/>
+      <c r="G2" s="78"/>
+      <c r="H2" s="78"/>
+      <c r="I2" s="78"/>
+      <c r="J2" s="78"/>
+      <c r="K2" s="78"/>
+      <c r="L2" s="78"/>
+      <c r="M2" s="78"/>
+      <c r="N2" s="78"/>
+      <c r="O2" s="78"/>
+      <c r="P2" s="78"/>
+      <c r="Q2" s="78"/>
+      <c r="R2" s="78"/>
+      <c r="S2" s="78"/>
+      <c r="T2" s="78"/>
+      <c r="U2" s="78"/>
+      <c r="V2" s="78"/>
+      <c r="W2" s="78"/>
+      <c r="X2" s="78"/>
+      <c r="Y2" s="78"/>
+      <c r="AU2" s="91" t="s">
         <v>77</v>
       </c>
-      <c r="AV2" s="75"/>
-      <c r="AW2" s="75"/>
-      <c r="AX2" s="76"/>
-      <c r="AY2" s="74" t="s">
+      <c r="AV2" s="92"/>
+      <c r="AW2" s="92"/>
+      <c r="AX2" s="93"/>
+      <c r="AY2" s="91" t="s">
         <v>14</v>
       </c>
-      <c r="AZ2" s="75"/>
-      <c r="BA2" s="76"/>
-      <c r="BB2" s="74" t="s">
+      <c r="AZ2" s="92"/>
+      <c r="BA2" s="93"/>
+      <c r="BB2" s="91" t="s">
         <v>59</v>
       </c>
-      <c r="BC2" s="75"/>
-      <c r="BD2" s="75"/>
-      <c r="BE2" s="75"/>
-      <c r="BF2" s="75"/>
-      <c r="BG2" s="76"/>
-      <c r="BH2" s="74" t="s">
+      <c r="BC2" s="92"/>
+      <c r="BD2" s="92"/>
+      <c r="BE2" s="92"/>
+      <c r="BF2" s="92"/>
+      <c r="BG2" s="93"/>
+      <c r="BH2" s="91" t="s">
         <v>60</v>
       </c>
-      <c r="BI2" s="75"/>
-      <c r="BJ2" s="76"/>
-      <c r="BK2" s="74" t="s">
+      <c r="BI2" s="92"/>
+      <c r="BJ2" s="93"/>
+      <c r="BK2" s="91" t="s">
         <v>61</v>
       </c>
-      <c r="BL2" s="75"/>
-      <c r="BM2" s="76"/>
+      <c r="BL2" s="92"/>
+      <c r="BM2" s="93"/>
     </row>
     <row r="3" spans="2:65" x14ac:dyDescent="0.25">
       <c r="B3" s="16"/>
       <c r="C3" s="24"/>
-      <c r="D3" s="63" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="63"/>
-      <c r="F3" s="63"/>
+      <c r="D3" s="80" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
       <c r="G3" s="20"/>
-      <c r="H3" s="59" t="s">
+      <c r="H3" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="59"/>
-      <c r="J3" s="59"/>
-      <c r="K3" s="59" t="s">
+      <c r="I3" s="76"/>
+      <c r="J3" s="76"/>
+      <c r="K3" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="L3" s="59"/>
-      <c r="M3" s="59"/>
-      <c r="N3" s="59" t="s">
+      <c r="L3" s="76"/>
+      <c r="M3" s="76"/>
+      <c r="N3" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="O3" s="59"/>
-      <c r="P3" s="59"/>
-      <c r="Q3" s="59" t="s">
+      <c r="O3" s="76"/>
+      <c r="P3" s="76"/>
+      <c r="Q3" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="R3" s="59"/>
-      <c r="S3" s="59"/>
-      <c r="T3" s="59" t="s">
+      <c r="R3" s="76"/>
+      <c r="S3" s="76"/>
+      <c r="T3" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="U3" s="59"/>
-      <c r="V3" s="59"/>
-      <c r="W3" s="59" t="s">
+      <c r="U3" s="76"/>
+      <c r="V3" s="76"/>
+      <c r="W3" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="X3" s="59"/>
-      <c r="Y3" s="59"/>
+      <c r="X3" s="76"/>
+      <c r="Y3" s="76"/>
       <c r="AA3" s="4" t="s">
         <v>38</v>
       </c>
@@ -28440,32 +28440,32 @@
       </c>
     </row>
     <row r="10" spans="2:65" ht="15" x14ac:dyDescent="0.25">
-      <c r="B10" s="61" t="s">
+      <c r="B10" s="78" t="s">
         <v>79</v>
       </c>
-      <c r="C10" s="61"/>
-      <c r="D10" s="61"/>
-      <c r="E10" s="61"/>
-      <c r="F10" s="61"/>
-      <c r="G10" s="61"/>
-      <c r="H10" s="61"/>
-      <c r="I10" s="61"/>
-      <c r="J10" s="61"/>
-      <c r="K10" s="61"/>
-      <c r="L10" s="61"/>
-      <c r="M10" s="61"/>
-      <c r="N10" s="61"/>
-      <c r="O10" s="61"/>
-      <c r="P10" s="61"/>
-      <c r="Q10" s="61"/>
-      <c r="R10" s="61"/>
-      <c r="S10" s="61"/>
-      <c r="T10" s="61"/>
-      <c r="U10" s="61"/>
-      <c r="V10" s="61"/>
-      <c r="W10" s="61"/>
-      <c r="X10" s="61"/>
-      <c r="Y10" s="61"/>
+      <c r="C10" s="78"/>
+      <c r="D10" s="78"/>
+      <c r="E10" s="78"/>
+      <c r="F10" s="78"/>
+      <c r="G10" s="78"/>
+      <c r="H10" s="78"/>
+      <c r="I10" s="78"/>
+      <c r="J10" s="78"/>
+      <c r="K10" s="78"/>
+      <c r="L10" s="78"/>
+      <c r="M10" s="78"/>
+      <c r="N10" s="78"/>
+      <c r="O10" s="78"/>
+      <c r="P10" s="78"/>
+      <c r="Q10" s="78"/>
+      <c r="R10" s="78"/>
+      <c r="S10" s="78"/>
+      <c r="T10" s="78"/>
+      <c r="U10" s="78"/>
+      <c r="V10" s="78"/>
+      <c r="W10" s="78"/>
+      <c r="X10" s="78"/>
+      <c r="Y10" s="78"/>
       <c r="AU10" s="31">
         <v>7</v>
       </c>
@@ -28544,42 +28544,42 @@
     <row r="11" spans="2:65" x14ac:dyDescent="0.25">
       <c r="B11" s="16"/>
       <c r="C11" s="24"/>
-      <c r="D11" s="63" t="s">
-        <v>3</v>
-      </c>
-      <c r="E11" s="63"/>
-      <c r="F11" s="63"/>
+      <c r="D11" s="80" t="s">
+        <v>3</v>
+      </c>
+      <c r="E11" s="80"/>
+      <c r="F11" s="80"/>
       <c r="G11" s="20"/>
-      <c r="H11" s="59" t="s">
+      <c r="H11" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="I11" s="59"/>
-      <c r="J11" s="59"/>
-      <c r="K11" s="59" t="s">
+      <c r="I11" s="76"/>
+      <c r="J11" s="76"/>
+      <c r="K11" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="L11" s="59"/>
-      <c r="M11" s="59"/>
-      <c r="N11" s="59" t="s">
+      <c r="L11" s="76"/>
+      <c r="M11" s="76"/>
+      <c r="N11" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="O11" s="59"/>
-      <c r="P11" s="59"/>
-      <c r="Q11" s="59" t="s">
+      <c r="O11" s="76"/>
+      <c r="P11" s="76"/>
+      <c r="Q11" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="R11" s="59"/>
-      <c r="S11" s="59"/>
-      <c r="T11" s="59" t="s">
+      <c r="R11" s="76"/>
+      <c r="S11" s="76"/>
+      <c r="T11" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="U11" s="59"/>
-      <c r="V11" s="59"/>
-      <c r="W11" s="59" t="s">
+      <c r="U11" s="76"/>
+      <c r="V11" s="76"/>
+      <c r="W11" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="X11" s="59"/>
-      <c r="Y11" s="59"/>
+      <c r="X11" s="76"/>
+      <c r="Y11" s="76"/>
       <c r="AA11" s="4" t="s">
         <v>38</v>
       </c>
@@ -28720,30 +28720,46 @@
         <f>IF(AB4=0,"Vencedor Q1",AB4)</f>
         <v>Itália</v>
       </c>
-      <c r="D12" s="56"/>
+      <c r="D12" s="56">
+        <v>3</v>
+      </c>
       <c r="E12" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F12" s="34"/>
+      <c r="F12" s="34">
+        <v>0</v>
+      </c>
       <c r="G12" s="21" t="str">
         <f>IF(AB5=0,"Vencedor Q4",AB5)</f>
         <v>Polônia</v>
       </c>
-      <c r="H12" s="33"/>
+      <c r="H12" s="33">
+        <v>25</v>
+      </c>
       <c r="I12" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="J12" s="34"/>
-      <c r="K12" s="33"/>
+      <c r="J12" s="34">
+        <v>18</v>
+      </c>
+      <c r="K12" s="33">
+        <v>25</v>
+      </c>
       <c r="L12" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="M12" s="34"/>
-      <c r="N12" s="33"/>
+      <c r="M12" s="34">
+        <v>16</v>
+      </c>
+      <c r="N12" s="33">
+        <v>25</v>
+      </c>
       <c r="O12" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="P12" s="34"/>
+      <c r="P12" s="34">
+        <v>14</v>
+      </c>
       <c r="Q12" s="33"/>
       <c r="R12" s="11" t="s">
         <v>6</v>
@@ -28756,30 +28772,30 @@
       <c r="V12" s="34"/>
       <c r="W12" s="12">
         <f>SUM(H12,K12,N12,Q12,T12)</f>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="X12" s="13" t="s">
         <v>6</v>
       </c>
       <c r="Y12" s="14">
         <f>SUM(J12,M12,P12,S12,V12)</f>
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="AA12" s="4">
         <f>AD12+AE12</f>
-        <v>0</v>
-      </c>
-      <c r="AB12" s="4">
+        <v>3</v>
+      </c>
+      <c r="AB12" s="4" t="str">
         <f>IF(OR(D12="",F12=""),0,IF(D12&gt;F12,C12,G12))</f>
-        <v>0</v>
+        <v>Itália</v>
       </c>
       <c r="AC12" s="4">
         <f>IF(OR(D12="",F12=""),0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD12" s="4">
         <f>IF(OR(D12="",F12=""),0,IF(D12&gt;F12,D12,F12))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AE12" s="4">
         <f>IF(OR(D12="",F12=""),0,IF(D12&gt;F12,F12,D12))</f>
@@ -28787,7 +28803,7 @@
       </c>
       <c r="AF12" s="4">
         <f>IF(AND(AD12=3,AE12=0),1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG12" s="4">
         <f>IF(AND(AD12=3,AE12=1),1,0)</f>
@@ -28799,19 +28815,19 @@
       </c>
       <c r="AI12" s="4">
         <f>IF(D12&gt;F12,SUM(H12,K12,N12,Q12,T12,),SUM(J12,M12,P12,S12,V12))</f>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="AJ12" s="4">
         <f>IF(D12&gt;F12,SUM(J12,M12,P12,S12,V12),SUM(H12,K12,N12,Q12,T12))</f>
-        <v>0</v>
-      </c>
-      <c r="AL12" s="4">
+        <v>48</v>
+      </c>
+      <c r="AL12" s="4" t="str">
         <f>IF(OR(D12="",F12=""),0,IF(D12&lt;F12,C12,G12))</f>
-        <v>0</v>
+        <v>Polônia</v>
       </c>
       <c r="AM12" s="4">
         <f>IF(OR(D12="",F12=""),0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN12" s="4">
         <f>IF(OR(D12="",F12=""),0,IF(D12&lt;F12,D12,F12))</f>
@@ -28819,7 +28835,7 @@
       </c>
       <c r="AO12" s="4">
         <f>IF(OR(D12="",F12=""),0,IF(D12&lt;F12,F12,D12))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AP12" s="4">
         <f>IF(AND(AN12=2,AO12=3),1,0)</f>
@@ -28831,15 +28847,15 @@
       </c>
       <c r="AR12" s="4">
         <f>IF(AND(AN12=0,AO12=3),1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS12" s="4">
         <f>IF(D12&lt;F12,SUM(H12,K12,N12,Q12,T12,),SUM(J12,M12,P12,S12,V12))</f>
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="AT12" s="4">
         <f>IF(D12&lt;F12,SUM(J12,M12,P12,S12,V12),SUM(H12,K12,N12,Q12,T12))</f>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="AU12" s="31">
         <v>9</v>
@@ -28924,70 +28940,94 @@
         <f>IF(AB6=0,"Vencedor Q2",AB6)</f>
         <v>Brasil</v>
       </c>
-      <c r="D13" s="56"/>
+      <c r="D13" s="56">
+        <v>3</v>
+      </c>
       <c r="E13" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F13" s="34"/>
+      <c r="F13" s="34">
+        <v>2</v>
+      </c>
       <c r="G13" s="21" t="str">
         <f>IF(AB7=0,"Vencedor Q3",AB7)</f>
         <v>Japão</v>
       </c>
-      <c r="H13" s="33"/>
+      <c r="H13" s="33">
+        <v>23</v>
+      </c>
       <c r="I13" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="J13" s="34"/>
-      <c r="K13" s="33"/>
+      <c r="J13" s="34">
+        <v>25</v>
+      </c>
+      <c r="K13" s="33">
+        <v>25</v>
+      </c>
       <c r="L13" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="M13" s="34"/>
-      <c r="N13" s="33"/>
+      <c r="M13" s="34">
+        <v>21</v>
+      </c>
+      <c r="N13" s="33">
+        <v>25</v>
+      </c>
       <c r="O13" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="P13" s="34"/>
-      <c r="Q13" s="33"/>
+      <c r="P13" s="34">
+        <v>18</v>
+      </c>
+      <c r="Q13" s="33">
+        <v>19</v>
+      </c>
       <c r="R13" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="S13" s="34"/>
-      <c r="T13" s="33"/>
+      <c r="S13" s="34">
+        <v>25</v>
+      </c>
+      <c r="T13" s="33">
+        <v>15</v>
+      </c>
       <c r="U13" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="V13" s="34"/>
+      <c r="V13" s="34">
+        <v>8</v>
+      </c>
       <c r="W13" s="12">
         <f>SUM(H13,K13,N13,Q13,T13)</f>
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="X13" s="13" t="s">
         <v>6</v>
       </c>
       <c r="Y13" s="14">
         <f>SUM(J13,M13,P13,S13,V13)</f>
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="AA13" s="4">
         <f>AD13+AE13</f>
-        <v>0</v>
-      </c>
-      <c r="AB13" s="4">
+        <v>5</v>
+      </c>
+      <c r="AB13" s="4" t="str">
         <f>IF(OR(D13="",F13=""),0,IF(D13&gt;F13,C13,G13))</f>
-        <v>0</v>
+        <v>Brasil</v>
       </c>
       <c r="AC13" s="4">
         <f>IF(OR(D13="",F13=""),0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD13" s="4">
         <f>IF(OR(D13="",F13=""),0,IF(D13&gt;F13,D13,F13))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AE13" s="4">
         <f>IF(OR(D13="",F13=""),0,IF(D13&gt;F13,F13,D13))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF13" s="4">
         <f>IF(AND(AD13=3,AE13=0),1,0)</f>
@@ -28999,35 +29039,35 @@
       </c>
       <c r="AH13" s="4">
         <f>IF(AND(AD13=3,AE13=2),1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI13" s="4">
         <f>IF(D13&gt;F13,SUM(H13,K13,N13,Q13,T13,),SUM(J13,M13,P13,S13,V13))</f>
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="AJ13" s="4">
         <f>IF(D13&gt;F13,SUM(J13,M13,P13,S13,V13),SUM(H13,K13,N13,Q13,T13))</f>
-        <v>0</v>
-      </c>
-      <c r="AL13" s="4">
+        <v>97</v>
+      </c>
+      <c r="AL13" s="4" t="str">
         <f>IF(OR(D13="",F13=""),0,IF(D13&lt;F13,C13,G13))</f>
-        <v>0</v>
+        <v>Japão</v>
       </c>
       <c r="AM13" s="4">
         <f>IF(OR(D13="",F13=""),0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN13" s="4">
         <f>IF(OR(D13="",F13=""),0,IF(D13&lt;F13,D13,F13))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AO13" s="4">
         <f>IF(OR(D13="",F13=""),0,IF(D13&lt;F13,F13,D13))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AP13" s="4">
         <f>IF(AND(AN13=2,AO13=3),1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ13" s="4">
         <f>IF(AND(AN13=1,AO13=3),1,0)</f>
@@ -29039,11 +29079,11 @@
       </c>
       <c r="AS13" s="4">
         <f>IF(D13&lt;F13,SUM(H13,K13,N13,Q13,T13,),SUM(J13,M13,P13,S13,V13))</f>
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="AT13" s="4">
         <f>IF(D13&lt;F13,SUM(J13,M13,P13,S13,V13),SUM(H13,K13,N13,Q13,T13))</f>
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="AU13" s="31">
         <v>10</v>
@@ -29349,32 +29389,32 @@
       </c>
     </row>
     <row r="17" spans="2:65" ht="15" x14ac:dyDescent="0.25">
-      <c r="B17" s="61" t="s">
+      <c r="B17" s="78" t="s">
         <v>80</v>
       </c>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="61"/>
-      <c r="F17" s="61"/>
-      <c r="G17" s="61"/>
-      <c r="H17" s="61"/>
-      <c r="I17" s="61"/>
-      <c r="J17" s="61"/>
-      <c r="K17" s="61"/>
-      <c r="L17" s="61"/>
-      <c r="M17" s="61"/>
-      <c r="N17" s="61"/>
-      <c r="O17" s="61"/>
-      <c r="P17" s="61"/>
-      <c r="Q17" s="61"/>
-      <c r="R17" s="61"/>
-      <c r="S17" s="61"/>
-      <c r="T17" s="61"/>
-      <c r="U17" s="61"/>
-      <c r="V17" s="61"/>
-      <c r="W17" s="61"/>
-      <c r="X17" s="61"/>
-      <c r="Y17" s="61"/>
+      <c r="C17" s="78"/>
+      <c r="D17" s="78"/>
+      <c r="E17" s="78"/>
+      <c r="F17" s="78"/>
+      <c r="G17" s="78"/>
+      <c r="H17" s="78"/>
+      <c r="I17" s="78"/>
+      <c r="J17" s="78"/>
+      <c r="K17" s="78"/>
+      <c r="L17" s="78"/>
+      <c r="M17" s="78"/>
+      <c r="N17" s="78"/>
+      <c r="O17" s="78"/>
+      <c r="P17" s="78"/>
+      <c r="Q17" s="78"/>
+      <c r="R17" s="78"/>
+      <c r="S17" s="78"/>
+      <c r="T17" s="78"/>
+      <c r="U17" s="78"/>
+      <c r="V17" s="78"/>
+      <c r="W17" s="78"/>
+      <c r="X17" s="78"/>
+      <c r="Y17" s="78"/>
       <c r="AA17" s="4" t="s">
         <v>38</v>
       </c>
@@ -29510,61 +29550,61 @@
     <row r="18" spans="2:65" x14ac:dyDescent="0.25">
       <c r="B18" s="16"/>
       <c r="C18" s="24"/>
-      <c r="D18" s="63" t="s">
-        <v>3</v>
-      </c>
-      <c r="E18" s="63"/>
-      <c r="F18" s="63"/>
+      <c r="D18" s="80" t="s">
+        <v>3</v>
+      </c>
+      <c r="E18" s="80"/>
+      <c r="F18" s="80"/>
       <c r="G18" s="20"/>
-      <c r="H18" s="59" t="s">
+      <c r="H18" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="I18" s="59"/>
-      <c r="J18" s="59"/>
-      <c r="K18" s="59" t="s">
+      <c r="I18" s="76"/>
+      <c r="J18" s="76"/>
+      <c r="K18" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="L18" s="59"/>
-      <c r="M18" s="59"/>
-      <c r="N18" s="59" t="s">
+      <c r="L18" s="76"/>
+      <c r="M18" s="76"/>
+      <c r="N18" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="O18" s="59"/>
-      <c r="P18" s="59"/>
-      <c r="Q18" s="59" t="s">
+      <c r="O18" s="76"/>
+      <c r="P18" s="76"/>
+      <c r="Q18" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="R18" s="59"/>
-      <c r="S18" s="59"/>
-      <c r="T18" s="59" t="s">
+      <c r="R18" s="76"/>
+      <c r="S18" s="76"/>
+      <c r="T18" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="U18" s="59"/>
-      <c r="V18" s="59"/>
-      <c r="W18" s="59" t="s">
+      <c r="U18" s="76"/>
+      <c r="V18" s="76"/>
+      <c r="W18" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="X18" s="59"/>
-      <c r="Y18" s="59"/>
+      <c r="X18" s="76"/>
+      <c r="Y18" s="76"/>
       <c r="AA18" s="4">
         <f>AD18+AE18</f>
-        <v>0</v>
-      </c>
-      <c r="AB18" s="4">
+        <v>4</v>
+      </c>
+      <c r="AB18" s="4" t="str">
         <f>IF(OR(D19="",F19=""),0,IF(D19&gt;F19,C19,G19))</f>
-        <v>0</v>
+        <v>Polônia</v>
       </c>
       <c r="AC18" s="4">
         <f>IF(OR(D19="",F19=""),0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD18" s="4">
         <f>IF(OR(D19="",F19=""),0,IF(D19&gt;F19,D19,F19))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AE18" s="4">
         <f>IF(OR(D19="",F19=""),0,IF(D19&gt;F19,F19,D19))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF18" s="4">
         <f>IF(AND(AD18=3,AE18=0),1,0)</f>
@@ -29572,7 +29612,7 @@
       </c>
       <c r="AG18" s="4">
         <f>IF(AND(AD18=3,AE18=1),1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH18" s="4">
         <f>IF(AND(AD18=3,AE18=2),1,0)</f>
@@ -29580,27 +29620,27 @@
       </c>
       <c r="AI18" s="4">
         <f>IF(D19&gt;F19,SUM(H19,K19,N19,Q19,T19,),SUM(J19,M19,P19,S19,V19))</f>
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="AJ18" s="4">
         <f>IF(D19&gt;F19,SUM(J19,M19,P19,S19,V19),SUM(H19,K19,N19,Q19,T19))</f>
-        <v>0</v>
-      </c>
-      <c r="AL18" s="4">
+        <v>80</v>
+      </c>
+      <c r="AL18" s="4" t="str">
         <f>IF(OR(D19="",F19=""),0,IF(D19&lt;F19,C19,G19))</f>
-        <v>0</v>
+        <v>Japão</v>
       </c>
       <c r="AM18" s="4">
         <f>IF(OR(D19="",F19=""),0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN18" s="4">
         <f>IF(OR(D19="",F19=""),0,IF(D19&lt;F19,D19,F19))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO18" s="4">
         <f>IF(OR(D19="",F19=""),0,IF(D19&lt;F19,F19,D19))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AP18" s="4">
         <f>IF(AND(AN18=2,AO18=3),1,0)</f>
@@ -29608,7 +29648,7 @@
       </c>
       <c r="AQ18" s="4">
         <f>IF(AND(AN18=1,AO18=3),1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR18" s="4">
         <f>IF(AND(AN18=0,AO18=3),1,0)</f>
@@ -29616,11 +29656,11 @@
       </c>
       <c r="AS18" s="4">
         <f>IF(D19&lt;F19,SUM(H19,K19,N19,Q19,T19,),SUM(J19,M19,P19,S19,V19))</f>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="AT18" s="4">
         <f>IF(D19&lt;F19,SUM(J19,M19,P19,S19,V19),SUM(H19,K19,N19,Q19,T19))</f>
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="AU18" s="31">
         <v>15</v>
@@ -29703,37 +29743,57 @@
       </c>
       <c r="C19" s="25" t="str">
         <f>IF(AL12=0,"Perdedor S1",AL12)</f>
-        <v>Perdedor S1</v>
-      </c>
-      <c r="D19" s="56"/>
+        <v>Polônia</v>
+      </c>
+      <c r="D19" s="56">
+        <v>3</v>
+      </c>
       <c r="E19" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F19" s="34"/>
+      <c r="F19" s="34">
+        <v>1</v>
+      </c>
       <c r="G19" s="21" t="str">
         <f>IF(AL13=0,"Perdedor S2",AL13)</f>
-        <v>Perdedor S2</v>
-      </c>
-      <c r="H19" s="33"/>
+        <v>Japão</v>
+      </c>
+      <c r="H19" s="33">
+        <v>25</v>
+      </c>
       <c r="I19" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="J19" s="34"/>
-      <c r="K19" s="33"/>
+      <c r="J19" s="34">
+        <v>15</v>
+      </c>
+      <c r="K19" s="33">
+        <v>24</v>
+      </c>
       <c r="L19" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="M19" s="34"/>
-      <c r="N19" s="33"/>
+      <c r="M19" s="34">
+        <v>26</v>
+      </c>
+      <c r="N19" s="33">
+        <v>25</v>
+      </c>
       <c r="O19" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="P19" s="34"/>
-      <c r="Q19" s="33"/>
+      <c r="P19" s="34">
+        <v>16</v>
+      </c>
+      <c r="Q19" s="33">
+        <v>25</v>
+      </c>
       <c r="R19" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="S19" s="34"/>
+      <c r="S19" s="34">
+        <v>23</v>
+      </c>
       <c r="T19" s="33"/>
       <c r="U19" s="11" t="s">
         <v>6</v>
@@ -29741,14 +29801,14 @@
       <c r="V19" s="34"/>
       <c r="W19" s="12">
         <f>SUM(H19,K19,N19,Q19,T19)</f>
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="X19" s="13" t="s">
         <v>6</v>
       </c>
       <c r="Y19" s="14">
         <f>SUM(J19,M19,P19,S19,V19)</f>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="AU19" s="31">
         <v>16</v>
@@ -29984,32 +30044,32 @@
       </c>
     </row>
     <row r="23" spans="2:65" ht="15" x14ac:dyDescent="0.25">
-      <c r="B23" s="61" t="s">
+      <c r="B23" s="78" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="61"/>
-      <c r="D23" s="61"/>
-      <c r="E23" s="61"/>
-      <c r="F23" s="61"/>
-      <c r="G23" s="61"/>
-      <c r="H23" s="61"/>
-      <c r="I23" s="61"/>
-      <c r="J23" s="61"/>
-      <c r="K23" s="61"/>
-      <c r="L23" s="61"/>
-      <c r="M23" s="61"/>
-      <c r="N23" s="61"/>
-      <c r="O23" s="61"/>
-      <c r="P23" s="61"/>
-      <c r="Q23" s="61"/>
-      <c r="R23" s="61"/>
-      <c r="S23" s="61"/>
-      <c r="T23" s="61"/>
-      <c r="U23" s="61"/>
-      <c r="V23" s="61"/>
-      <c r="W23" s="61"/>
-      <c r="X23" s="61"/>
-      <c r="Y23" s="61"/>
+      <c r="C23" s="78"/>
+      <c r="D23" s="78"/>
+      <c r="E23" s="78"/>
+      <c r="F23" s="78"/>
+      <c r="G23" s="78"/>
+      <c r="H23" s="78"/>
+      <c r="I23" s="78"/>
+      <c r="J23" s="78"/>
+      <c r="K23" s="78"/>
+      <c r="L23" s="78"/>
+      <c r="M23" s="78"/>
+      <c r="N23" s="78"/>
+      <c r="O23" s="78"/>
+      <c r="P23" s="78"/>
+      <c r="Q23" s="78"/>
+      <c r="R23" s="78"/>
+      <c r="S23" s="78"/>
+      <c r="T23" s="78"/>
+      <c r="U23" s="78"/>
+      <c r="V23" s="78"/>
+      <c r="W23" s="78"/>
+      <c r="X23" s="78"/>
+      <c r="Y23" s="78"/>
       <c r="AA23" s="4" t="s">
         <v>38</v>
       </c>
@@ -30067,70 +30127,70 @@
       <c r="AT23" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="AU23" s="73" t="s">
+      <c r="AU23" s="90" t="s">
         <v>87</v>
       </c>
-      <c r="AV23" s="73"/>
-      <c r="AW23" s="84"/>
+      <c r="AV23" s="90"/>
+      <c r="AW23" s="62"/>
     </row>
     <row r="24" spans="2:65" x14ac:dyDescent="0.25">
       <c r="B24" s="16"/>
       <c r="C24" s="24"/>
-      <c r="D24" s="63" t="s">
-        <v>3</v>
-      </c>
-      <c r="E24" s="63"/>
-      <c r="F24" s="63"/>
+      <c r="D24" s="80" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" s="80"/>
+      <c r="F24" s="80"/>
       <c r="G24" s="20"/>
-      <c r="H24" s="59" t="s">
+      <c r="H24" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="I24" s="59"/>
-      <c r="J24" s="59"/>
-      <c r="K24" s="59" t="s">
+      <c r="I24" s="76"/>
+      <c r="J24" s="76"/>
+      <c r="K24" s="76" t="s">
         <v>5</v>
       </c>
-      <c r="L24" s="59"/>
-      <c r="M24" s="59"/>
-      <c r="N24" s="59" t="s">
+      <c r="L24" s="76"/>
+      <c r="M24" s="76"/>
+      <c r="N24" s="76" t="s">
         <v>7</v>
       </c>
-      <c r="O24" s="59"/>
-      <c r="P24" s="59"/>
-      <c r="Q24" s="59" t="s">
+      <c r="O24" s="76"/>
+      <c r="P24" s="76"/>
+      <c r="Q24" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="R24" s="59"/>
-      <c r="S24" s="59"/>
-      <c r="T24" s="59" t="s">
+      <c r="R24" s="76"/>
+      <c r="S24" s="76"/>
+      <c r="T24" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="U24" s="59"/>
-      <c r="V24" s="59"/>
-      <c r="W24" s="59" t="s">
+      <c r="U24" s="76"/>
+      <c r="V24" s="76"/>
+      <c r="W24" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="X24" s="59"/>
-      <c r="Y24" s="59"/>
+      <c r="X24" s="76"/>
+      <c r="Y24" s="76"/>
       <c r="AA24" s="4">
         <f>AD24+AE24</f>
-        <v>0</v>
-      </c>
-      <c r="AB24" s="4">
+        <v>4</v>
+      </c>
+      <c r="AB24" s="4" t="str">
         <f>IF(OR(D25="",F25=""),0,IF(D25&gt;F25,C25,G25))</f>
-        <v>0</v>
+        <v>Itália</v>
       </c>
       <c r="AC24" s="4">
         <f>IF(OR(D25="",F25=""),0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD24" s="4">
         <f>IF(OR(D25="",F25=""),0,IF(D25&gt;F25,D25,F25))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AE24" s="4">
         <f>IF(OR(D25="",F25=""),0,IF(D25&gt;F25,F25,D25))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF24" s="4">
         <f>IF(AND(AD24=3,AE24=0),1,0)</f>
@@ -30138,7 +30198,7 @@
       </c>
       <c r="AG24" s="4">
         <f>IF(AND(AD24=3,AE24=1),1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH24" s="4">
         <f>IF(AND(AD24=3,AE24=2),1,0)</f>
@@ -30146,27 +30206,27 @@
       </c>
       <c r="AI24" s="4">
         <f>IF(D25&gt;F25,SUM(H25,K25,N25,Q25,T25,),SUM(J25,M25,P25,S25,V25))</f>
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="AJ24" s="4">
         <f>IF(D25&gt;F25,SUM(J25,M25,P25,S25,V25),SUM(H25,K25,N25,Q25,T25))</f>
-        <v>0</v>
-      </c>
-      <c r="AL24" s="4">
+        <v>87</v>
+      </c>
+      <c r="AL24" s="4" t="str">
         <f>IF(OR(D25="",F25=""),0,IF(D25&lt;F25,C25,G25))</f>
-        <v>0</v>
+        <v>Brasil</v>
       </c>
       <c r="AM24" s="4">
         <f>IF(OR(D25="",F25=""),0,1)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN24" s="4">
         <f>IF(OR(D25="",F25=""),0,IF(D25&lt;F25,D25,F25))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO24" s="4">
         <f>IF(OR(D25="",F25=""),0,IF(D25&lt;F25,F25,D25))</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AP24" s="4">
         <f>IF(AND(AN24=2,AO24=3),1,0)</f>
@@ -30174,7 +30234,7 @@
       </c>
       <c r="AQ24" s="4">
         <f>IF(AND(AN24=1,AO24=3),1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR24" s="4">
         <f>IF(AND(AN24=0,AO24=3),1,0)</f>
@@ -30182,17 +30242,17 @@
       </c>
       <c r="AS24" s="4">
         <f>IF(D25&lt;F25,SUM(H25,K25,N25,Q25,T25,),SUM(J25,M25,P25,S25,V25))</f>
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="AT24" s="4">
         <f>IF(D25&lt;F25,SUM(J25,M25,P25,S25,V25),SUM(H25,K25,N25,Q25,T25))</f>
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="AU24" s="54"/>
       <c r="AV24" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="AW24" s="85"/>
+      <c r="AW24" s="63"/>
     </row>
     <row r="25" spans="2:65" x14ac:dyDescent="0.25">
       <c r="B25" s="17">
@@ -30200,37 +30260,57 @@
       </c>
       <c r="C25" s="25" t="str">
         <f>IF(AB12=0,"Vencedor S1",AB12)</f>
-        <v>Vencedor S1</v>
-      </c>
-      <c r="D25" s="56"/>
+        <v>Itália</v>
+      </c>
+      <c r="D25" s="56">
+        <v>3</v>
+      </c>
       <c r="E25" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="F25" s="34"/>
+      <c r="F25" s="34">
+        <v>1</v>
+      </c>
       <c r="G25" s="21" t="str">
         <f>IF(AB13=0,"Vencedor S2",AB13)</f>
-        <v>Vencedor S2</v>
-      </c>
-      <c r="H25" s="33"/>
+        <v>Brasil</v>
+      </c>
+      <c r="H25" s="33">
+        <v>22</v>
+      </c>
       <c r="I25" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="J25" s="34"/>
-      <c r="K25" s="33"/>
+      <c r="J25" s="34">
+        <v>25</v>
+      </c>
+      <c r="K25" s="33">
+        <v>25</v>
+      </c>
       <c r="L25" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="M25" s="34"/>
-      <c r="N25" s="33"/>
+      <c r="M25" s="34">
+        <v>18</v>
+      </c>
+      <c r="N25" s="33">
+        <v>25</v>
+      </c>
       <c r="O25" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="P25" s="34"/>
-      <c r="Q25" s="33"/>
+      <c r="P25" s="34">
+        <v>22</v>
+      </c>
+      <c r="Q25" s="33">
+        <v>25</v>
+      </c>
       <c r="R25" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="S25" s="34"/>
+      <c r="S25" s="34">
+        <v>22</v>
+      </c>
       <c r="T25" s="33"/>
       <c r="U25" s="11" t="s">
         <v>6</v>
@@ -30238,27 +30318,27 @@
       <c r="V25" s="34"/>
       <c r="W25" s="12">
         <f>SUM(H25,K25,N25,Q25,T25)</f>
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="X25" s="13" t="s">
         <v>6</v>
       </c>
       <c r="Y25" s="14">
         <f>SUM(J25,M25,P25,S25,V25)</f>
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="AU25" s="55"/>
       <c r="AV25" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="AW25" s="85"/>
+      <c r="AW25" s="63"/>
     </row>
     <row r="26" spans="2:65" x14ac:dyDescent="0.25">
       <c r="AU26" s="57"/>
       <c r="AV26" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="AW26" s="85"/>
+      <c r="AW26" s="63"/>
     </row>
     <row r="27" spans="2:65" s="39" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="19"/>
@@ -30287,10 +30367,10 @@
       <c r="Y27" s="4"/>
     </row>
     <row r="28" spans="2:65" s="41" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="79" t="s">
+      <c r="B28" s="96" t="s">
         <v>97</v>
       </c>
-      <c r="C28" s="79"/>
+      <c r="C28" s="96"/>
       <c r="D28" s="44"/>
       <c r="E28" s="39"/>
       <c r="F28" s="46"/>
@@ -30313,11 +30393,11 @@
       <c r="W28" s="39"/>
       <c r="X28" s="39"/>
       <c r="Y28" s="39"/>
-      <c r="AU28" s="77" t="s">
+      <c r="AU28" s="94" t="s">
         <v>91</v>
       </c>
-      <c r="AV28" s="78"/>
-      <c r="AW28" s="86"/>
+      <c r="AV28" s="95"/>
+      <c r="AW28" s="64"/>
     </row>
     <row r="29" spans="2:65" s="41" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="50" t="s">
@@ -30325,16 +30405,16 @@
       </c>
       <c r="C29" s="48" t="str">
         <f>IF(AB24=0,"Campeão",AB24)</f>
-        <v>Campeão</v>
+        <v>Itália</v>
       </c>
       <c r="D29" s="45"/>
       <c r="F29" s="47"/>
       <c r="G29" s="42"/>
-      <c r="AU29" s="64" t="s">
+      <c r="AU29" s="81" t="s">
         <v>92</v>
       </c>
-      <c r="AV29" s="65"/>
-      <c r="AW29" s="87"/>
+      <c r="AV29" s="82"/>
+      <c r="AW29" s="65"/>
     </row>
     <row r="30" spans="2:65" s="41" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="51" t="s">
@@ -30342,16 +30422,16 @@
       </c>
       <c r="C30" s="49" t="str">
         <f>IF(AL24=0,"Vice",AL24)</f>
-        <v>Vice</v>
+        <v>Brasil</v>
       </c>
       <c r="D30" s="45"/>
       <c r="F30" s="47"/>
       <c r="G30" s="42"/>
-      <c r="AU30" s="66" t="s">
+      <c r="AU30" s="83" t="s">
         <v>93</v>
       </c>
-      <c r="AV30" s="67"/>
-      <c r="AW30" s="88"/>
+      <c r="AV30" s="84"/>
+      <c r="AW30" s="66"/>
     </row>
     <row r="31" spans="2:65" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="52" t="s">
@@ -30359,7 +30439,7 @@
       </c>
       <c r="C31" s="49" t="str">
         <f>IF(AB18=0,"Terceiro",AB18)</f>
-        <v>Terceiro</v>
+        <v>Polônia</v>
       </c>
       <c r="D31" s="45"/>
       <c r="E31" s="41"/>
@@ -30383,45 +30463,45 @@
       <c r="W31" s="41"/>
       <c r="X31" s="41"/>
       <c r="Y31" s="41"/>
-      <c r="AU31" s="66" t="s">
+      <c r="AU31" s="83" t="s">
         <v>94</v>
       </c>
-      <c r="AV31" s="67"/>
-      <c r="AW31" s="88"/>
+      <c r="AV31" s="84"/>
+      <c r="AW31" s="66"/>
     </row>
     <row r="32" spans="2:65" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="81">
+      <c r="B32" s="59">
         <v>4</v>
       </c>
-      <c r="C32" s="96" t="str">
+      <c r="C32" s="74" t="str">
         <f>IF(AL18=0,"",AL18)</f>
-        <v/>
-      </c>
-      <c r="AU32" s="66" t="s">
+        <v>Japão</v>
+      </c>
+      <c r="AU32" s="83" t="s">
         <v>95</v>
       </c>
-      <c r="AV32" s="67"/>
-      <c r="AW32" s="88"/>
+      <c r="AV32" s="84"/>
+      <c r="AW32" s="66"/>
     </row>
     <row r="33" spans="2:49" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="83">
+      <c r="B33" s="61">
         <v>5</v>
       </c>
-      <c r="C33" s="95" t="str">
+      <c r="C33" s="73" t="str">
         <f>IFERROR(VLOOKUP(SMALL($AK$34:$AK$37,1),$AK$34:$AL$37,2,FALSE),"")</f>
         <v>China</v>
       </c>
-      <c r="AU33" s="68" t="s">
+      <c r="AU33" s="85" t="s">
         <v>96</v>
       </c>
-      <c r="AV33" s="69"/>
-      <c r="AW33" s="89"/>
+      <c r="AV33" s="86"/>
+      <c r="AW33" s="67"/>
     </row>
     <row r="34" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="B34" s="82">
-        <v>6</v>
-      </c>
-      <c r="C34" s="80" t="str">
+      <c r="B34" s="60">
+        <v>6</v>
+      </c>
+      <c r="C34" s="58" t="str">
         <f>IFERROR(VLOOKUP(SMALL($AK$34:$AK$37,2),$AK$34:$AL$37,2,FALSE),"")</f>
         <v>Turquia</v>
       </c>
@@ -30439,10 +30519,10 @@
       </c>
     </row>
     <row r="35" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="B35" s="82">
+      <c r="B35" s="60">
         <v>7</v>
       </c>
-      <c r="C35" s="80" t="str">
+      <c r="C35" s="58" t="str">
         <f>IFERROR(VLOOKUP(SMALL($AK$34:$AK$37,3),$AK$34:$AL$37,2,FALSE),"")</f>
         <v>Alemanha</v>
       </c>
@@ -30460,10 +30540,10 @@
       </c>
     </row>
     <row r="36" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="B36" s="82">
+      <c r="B36" s="60">
         <v>8</v>
       </c>
-      <c r="C36" s="80" t="str">
+      <c r="C36" s="58" t="str">
         <f>IFERROR(VLOOKUP(SMALL($AK$34:$AK$37,4),$AK$34:$AL$37,2,FALSE),"")</f>
         <v>Estados Unidos</v>
       </c>
@@ -30481,14 +30561,14 @@
       </c>
     </row>
     <row r="37" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="B37" s="82">
+      <c r="B37" s="60">
         <v>9</v>
       </c>
-      <c r="C37" s="80" t="str">
+      <c r="C37" s="58" t="str">
         <f>IF($AY$22&lt;216,"",VLOOKUP(B37-D37,$AU$4:AV$21,2,FALSE))</f>
         <v>França</v>
       </c>
-      <c r="D37" s="90">
+      <c r="D37" s="68">
         <f t="shared" ref="D37:D45" si="3">IF(B37&lt;=$G$50,1,0)</f>
         <v>0</v>
       </c>
@@ -30506,14 +30586,14 @@
       </c>
     </row>
     <row r="38" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="B38" s="82">
+      <c r="B38" s="60">
         <v>10</v>
       </c>
-      <c r="C38" s="80" t="str">
+      <c r="C38" s="58" t="str">
         <f>IF($AY$22&lt;216,"",VLOOKUP(B38-D38,$AU$4:AV$21,2,FALSE))</f>
         <v>Holanda</v>
       </c>
-      <c r="D38" s="90">
+      <c r="D38" s="68">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -30523,265 +30603,265 @@
       </c>
     </row>
     <row r="39" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="B39" s="82">
+      <c r="B39" s="60">
         <v>11</v>
       </c>
-      <c r="C39" s="80" t="str">
+      <c r="C39" s="58" t="str">
         <f>IF($AY$22&lt;216,"",VLOOKUP(B39-D39,$AU$4:AV$21,2,FALSE))</f>
         <v>República Tcheca</v>
       </c>
-      <c r="D39" s="90">
+      <c r="D39" s="68">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="G39" s="4"/>
     </row>
     <row r="40" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="B40" s="82">
+      <c r="B40" s="60">
         <v>12</v>
       </c>
-      <c r="C40" s="80" t="str">
+      <c r="C40" s="58" t="str">
         <f>IF($AY$22&lt;216,"",VLOOKUP(B40-D40,$AU$4:AV$21,2,FALSE))</f>
         <v>República Dominicana</v>
       </c>
-      <c r="D40" s="90">
+      <c r="D40" s="68">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="41" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="B41" s="82">
+      <c r="B41" s="60">
         <v>13</v>
       </c>
-      <c r="C41" s="80" t="str">
+      <c r="C41" s="58" t="str">
         <f>IF($AY$22&lt;216,"",VLOOKUP(B41-D41,$AU$4:AV$21,2,FALSE))</f>
         <v>Bulgária</v>
       </c>
-      <c r="D41" s="90">
+      <c r="D41" s="68">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="42" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="B42" s="82">
+      <c r="B42" s="60">
         <v>14</v>
       </c>
-      <c r="C42" s="80" t="str">
+      <c r="C42" s="58" t="str">
         <f>IF($AY$22&lt;216,"",VLOOKUP(B42-D42,$AU$4:AV$21,2,FALSE))</f>
         <v>Bélgica</v>
       </c>
-      <c r="D42" s="90">
+      <c r="D42" s="68">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="43" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="B43" s="82">
+      <c r="B43" s="60">
         <v>15</v>
       </c>
-      <c r="C43" s="80" t="str">
+      <c r="C43" s="58" t="str">
         <f>IF($AY$22&lt;216,"",VLOOKUP(B43-D43,$AU$4:AV$21,2,FALSE))</f>
         <v>Sérvia</v>
       </c>
-      <c r="D43" s="90">
+      <c r="D43" s="68">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="44" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="B44" s="82">
+      <c r="B44" s="60">
         <v>16</v>
       </c>
-      <c r="C44" s="80" t="str">
+      <c r="C44" s="58" t="str">
         <f>IF($AY$22&lt;216,"",VLOOKUP(B44-D44,$AU$4:AV$21,2,FALSE))</f>
         <v>Canadá</v>
       </c>
-      <c r="D44" s="90">
+      <c r="D44" s="68">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="45" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="B45" s="82">
+      <c r="B45" s="60">
         <v>17</v>
       </c>
-      <c r="C45" s="80" t="str">
+      <c r="C45" s="58" t="str">
         <f>IF($AY$22&lt;216,"",VLOOKUP(B45-D45,$AU$4:AV$21,2,FALSE))</f>
         <v>Tailândia</v>
       </c>
-      <c r="D45" s="90">
+      <c r="D45" s="68">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
     </row>
     <row r="46" spans="2:49" x14ac:dyDescent="0.25">
-      <c r="B46" s="82">
+      <c r="B46" s="60">
         <v>18</v>
       </c>
-      <c r="C46" s="80" t="str">
+      <c r="C46" s="58" t="str">
         <f>IF($AY$22&lt;216,"",VLOOKUP(B46-D46,$AU$4:AV$21,2,FALSE))</f>
         <v>Coreia do Sul</v>
       </c>
-      <c r="D46" s="90">
+      <c r="D46" s="68">
         <f>IF(B46&lt;=$G$50,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="50" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B50" s="91">
+      <c r="B50" s="69">
         <v>9</v>
       </c>
-      <c r="C50" s="92" t="str">
+      <c r="C50" s="70" t="str">
         <f t="shared" ref="C50:C58" si="4">IF($AY$22&lt;216,"",AV12)</f>
         <v>França</v>
       </c>
-      <c r="D50" s="90">
+      <c r="D50" s="68">
         <v>1</v>
       </c>
       <c r="E50" s="53"/>
-      <c r="F50" s="93">
+      <c r="F50" s="71">
         <f>SUMIF(C50:C59,Dummy!Z1,Finais!D50:D60)</f>
         <v>0</v>
       </c>
-      <c r="G50" s="94">
+      <c r="G50" s="72">
         <f>IF(F50=1,VLOOKUP(Dummy!Z1,AV4:AW21,2,FALSE),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="51" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B51" s="91">
+      <c r="B51" s="69">
         <v>10</v>
       </c>
-      <c r="C51" s="92" t="str">
+      <c r="C51" s="70" t="str">
         <f t="shared" si="4"/>
         <v>Holanda</v>
       </c>
-      <c r="D51" s="90">
+      <c r="D51" s="68">
         <v>1</v>
       </c>
       <c r="E51" s="53"/>
-      <c r="F51" s="93"/>
-      <c r="G51" s="94"/>
+      <c r="F51" s="71"/>
+      <c r="G51" s="72"/>
     </row>
     <row r="52" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B52" s="91">
+      <c r="B52" s="69">
         <v>11</v>
       </c>
-      <c r="C52" s="92" t="str">
+      <c r="C52" s="70" t="str">
         <f t="shared" si="4"/>
         <v>República Tcheca</v>
       </c>
-      <c r="D52" s="90">
+      <c r="D52" s="68">
         <v>1</v>
       </c>
       <c r="E52" s="53"/>
-      <c r="F52" s="93"/>
-      <c r="G52" s="94"/>
+      <c r="F52" s="71"/>
+      <c r="G52" s="72"/>
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B53" s="91">
+      <c r="B53" s="69">
         <v>12</v>
       </c>
-      <c r="C53" s="92" t="str">
+      <c r="C53" s="70" t="str">
         <f t="shared" si="4"/>
         <v>República Dominicana</v>
       </c>
-      <c r="D53" s="90">
+      <c r="D53" s="68">
         <v>1</v>
       </c>
       <c r="E53" s="53"/>
-      <c r="F53" s="93"/>
-      <c r="G53" s="94"/>
+      <c r="F53" s="71"/>
+      <c r="G53" s="72"/>
     </row>
     <row r="54" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B54" s="91">
+      <c r="B54" s="69">
         <v>13</v>
       </c>
-      <c r="C54" s="92" t="str">
+      <c r="C54" s="70" t="str">
         <f t="shared" si="4"/>
         <v>Bulgária</v>
       </c>
-      <c r="D54" s="90">
+      <c r="D54" s="68">
         <v>1</v>
       </c>
       <c r="E54" s="53"/>
-      <c r="F54" s="93"/>
-      <c r="G54" s="94"/>
+      <c r="F54" s="71"/>
+      <c r="G54" s="72"/>
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B55" s="91">
+      <c r="B55" s="69">
         <v>14</v>
       </c>
-      <c r="C55" s="92" t="str">
+      <c r="C55" s="70" t="str">
         <f t="shared" si="4"/>
         <v>Bélgica</v>
       </c>
-      <c r="D55" s="90">
+      <c r="D55" s="68">
         <v>1</v>
       </c>
       <c r="E55" s="53"/>
-      <c r="F55" s="93"/>
-      <c r="G55" s="94"/>
+      <c r="F55" s="71"/>
+      <c r="G55" s="72"/>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B56" s="91">
+      <c r="B56" s="69">
         <v>15</v>
       </c>
-      <c r="C56" s="92" t="str">
+      <c r="C56" s="70" t="str">
         <f t="shared" si="4"/>
         <v>Sérvia</v>
       </c>
-      <c r="D56" s="90">
+      <c r="D56" s="68">
         <v>1</v>
       </c>
       <c r="E56" s="53"/>
-      <c r="F56" s="93"/>
-      <c r="G56" s="94"/>
+      <c r="F56" s="71"/>
+      <c r="G56" s="72"/>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B57" s="91">
+      <c r="B57" s="69">
         <v>16</v>
       </c>
-      <c r="C57" s="92" t="str">
+      <c r="C57" s="70" t="str">
         <f t="shared" si="4"/>
         <v>Canadá</v>
       </c>
-      <c r="D57" s="90">
+      <c r="D57" s="68">
         <v>1</v>
       </c>
       <c r="E57" s="53"/>
-      <c r="F57" s="93"/>
-      <c r="G57" s="94"/>
+      <c r="F57" s="71"/>
+      <c r="G57" s="72"/>
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B58" s="91">
+      <c r="B58" s="69">
         <v>17</v>
       </c>
-      <c r="C58" s="92" t="str">
+      <c r="C58" s="70" t="str">
         <f t="shared" si="4"/>
         <v>Tailândia</v>
       </c>
-      <c r="D58" s="90">
+      <c r="D58" s="68">
         <v>1</v>
       </c>
       <c r="E58" s="53"/>
-      <c r="F58" s="93"/>
-      <c r="G58" s="94"/>
+      <c r="F58" s="71"/>
+      <c r="G58" s="72"/>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B59" s="91">
+      <c r="B59" s="69">
         <v>18</v>
       </c>
-      <c r="C59" s="92" t="str">
+      <c r="C59" s="70" t="str">
         <f>IF($AY$22&lt;216,"",AV21)</f>
         <v>Coreia do Sul</v>
       </c>
-      <c r="D59" s="90">
+      <c r="D59" s="68">
         <v>1</v>
       </c>
       <c r="E59" s="53"/>
-      <c r="F59" s="93"/>
-      <c r="G59" s="94"/>
+      <c r="F59" s="71"/>
+      <c r="G59" s="72"/>
     </row>
   </sheetData>
   <sheetProtection password="CC01" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
@@ -30858,72 +30938,72 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BN16:XFD16 BN21:XFD22 BN2:XFD10 BN12:XFD13 BN18:XFD18 BN24:XFD38 AU3:BM20 A1:XFD1 A16:A18 Z16:AT18 B17:Y19 B22:Y27 A43:A1048576 A21:A38 B28 D28:Y28 C36:Y36 C46:Y46 B36:B46 E44:Y45 E37:Y38 Z21:AT33 Z38:AT38 B29:Y35 AA34:AT37 Z43:XFD1048576 A2:AT13 B47:Y1048576 C37:D45">
-    <cfRule type="cellIs" dxfId="0" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="16" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BN11:XFD11">
-    <cfRule type="cellIs" dxfId="17" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="13" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BN17:XFD17">
-    <cfRule type="cellIs" dxfId="16" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="12" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="BN23:XFD23">
-    <cfRule type="cellIs" dxfId="15" priority="11" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="11" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AU2:BM2">
-    <cfRule type="cellIs" dxfId="14" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="7" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AV21:BM21">
-    <cfRule type="cellIs" dxfId="13" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="6" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AU21:BM21">
-    <cfRule type="expression" dxfId="12" priority="3">
+    <cfRule type="expression" dxfId="11" priority="3">
       <formula>$AY$22=216</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T25:V25 T19:V19">
-    <cfRule type="expression" dxfId="11" priority="88">
+    <cfRule type="expression" dxfId="10" priority="88">
       <formula>$AA18&lt;5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q25:S25 Q19:S19">
-    <cfRule type="expression" dxfId="10" priority="90">
+    <cfRule type="expression" dxfId="9" priority="90">
       <formula>$AA18&lt;4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N25:P25 N19:P19">
-    <cfRule type="expression" dxfId="9" priority="92">
+    <cfRule type="expression" dxfId="8" priority="92">
       <formula>$AA18&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25:M25 K19:M19">
-    <cfRule type="expression" dxfId="8" priority="94">
+    <cfRule type="expression" dxfId="7" priority="94">
       <formula>$AA18&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W19:Y19 H25:J25 W25:Y25 H19:J19">
-    <cfRule type="expression" dxfId="7" priority="96">
+    <cfRule type="expression" dxfId="6" priority="96">
       <formula>$AA18=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AU28:AU33">
-    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
       <formula>"Brasil"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C33:C36">
-    <cfRule type="expression" dxfId="1" priority="1">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$C33=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -31270,16 +31350,16 @@
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1C0F6A83-8A20-4128-AC08-526BDD0F4F5D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="dc8c2798-6aba-4af7-93a4-b89253b03650"/>
     <ds:schemaRef ds:uri="2c8c20e6-817c-474f-b9c2-eb2b1ac24837"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>